<commit_message>
remove bloat/commentary from the data dictionary. Keep them under 'Known data issues'.
</commit_message>
<xml_diff>
--- a/AnimalCollisionsWeather/dataRAW/data_dictionary_weather_population.xlsx
+++ b/AnimalCollisionsWeather/dataRAW/data_dictionary_weather_population.xlsx
@@ -486,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L127"/>
+  <dimension ref="A1:K115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -559,10 +559,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="72" customHeight="1">
+    <row r="2" ht="56" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>HOW TO USE THIS TAB: the weather and population pipelines (Wendy). One row per variable in each pipeline output, grouped by output file in column A -- the file name is written on the first row of each block only. Columns A-K match the DVC and wildlife dictionaries so the tabs can be stacked. Column I gives the Python construction and, where the variable reaches main_data_county_year.dta, the Stata step in build_main_data_county_year.do that puts it there. Column J says whether the variable survives into that .dta and under what name -- every monthly weather measure arrives as 12 columns, _m1 .. _m12. Unresolved issues are listed below the table.</t>
+          <t>HOW TO USE THIS TAB: the weather and population pipelines. One row per variable in each pipeline output, grouped by output file in column A -- the file name appears on the first row of each block. Column I gives the construction and, where the variable reaches main_data_county_year.dta, the step in build_main_data_county_year.do that puts it there; column J says under what name it arrives. Known data issues are listed below the table. Script-level design decisions live in codePYTHON/SCRIPT_OVERVIEW.md, not here.</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -590,7 +590,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>5-digit county FIPS (2-digit state + 3-digit county); the canonical merge key against every other RA's county-level panel</t>
+          <t>5-digit county FIPS (state + county); the merge key against every other county-level panel</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
@@ -610,7 +610,7 @@
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd via 02a_extract_prism_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
+          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
@@ -620,17 +620,17 @@
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>Written by the GEE extraction; imported into Stata with stringcols(1 2 3) so leading zeros survive</t>
+          <t>Imported with stringcols(1 2 3) so leading zeros survive</t>
         </is>
       </c>
       <c r="J3" s="5" t="inlineStr">
         <is>
-          <t>No (this file does not feed the merge)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K3" s="5" t="inlineStr">
         <is>
-          <t>Text, not numeric -- leading zeros are meaningful. Merge on geoid, never on county_name (names are not unique across states). County universe is TIGER/2018 everywhere in this pipeline. This file is the descriptive-exhibit panel (09a/09b), NOT the merge input -- SECTION 1 of build_main_data_county_year.do reads prism_derived_weather_vars.csv instead.</t>
+          <t>Text, not numeric. Merge on geoid, never on county_name. County universe is TIGER/2018 throughout. This file is the descriptive-exhibit panel (09a/09b), not the merge input -- SECTION 1 reads prism_derived_weather_vars.csv.</t>
         </is>
       </c>
     </row>
@@ -663,7 +663,7 @@
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>TIGER/2018/Counties (Earth Engine FeatureCollection), carried through the GEE extraction</t>
+          <t>TIGER/2018/Counties (Earth Engine FeatureCollection)</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
@@ -673,19 +673,15 @@
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>Carried through from the extraction; stringcols on import</t>
+          <t>Carried through from the extraction</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>No (this file does not feed the merge)</t>
-        </is>
-      </c>
-      <c r="K4" s="5" t="inlineStr">
-        <is>
-          <t>CONUS scope is defined once, in gee_extract_utils.CONUS_STATE_FIPS, and imported by every extraction script.</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="n"/>
@@ -716,7 +712,7 @@
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>TIGER/2018/Counties (Earth Engine FeatureCollection), carried through the GEE extraction</t>
+          <t>TIGER/2018/Counties (Earth Engine FeatureCollection)</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
@@ -726,19 +722,15 @@
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Carried through from the extraction; stringcols on import</t>
+          <t>Carried through from the extraction</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>No (this file does not feed the merge)</t>
-        </is>
-      </c>
-      <c r="K5" s="5" t="inlineStr">
-        <is>
-          <t>Combine with state_fips for a nationally unique key, or just use geoid.</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="n"/>
@@ -769,7 +761,7 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>TIGER/2018/Counties (Earth Engine FeatureCollection), carried through the GEE extraction</t>
+          <t>TIGER/2018/Counties (Earth Engine FeatureCollection)</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
@@ -784,12 +776,12 @@
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>No (this file does not feed the merge)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t>Reference/QA only -- not unique across states, so never a merge key.</t>
+          <t>Reference only -- not unique across states, so never a merge key.</t>
         </is>
       </c>
     </row>
@@ -822,7 +814,7 @@
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Derived from the daily extraction date</t>
+          <t>Daily extraction date</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -832,7 +824,7 @@
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>Parsed from the daily `date` column during aggregation</t>
+          <t>Parsed from the daily date column</t>
         </is>
       </c>
       <c r="J7" s="5" t="inlineStr">
@@ -842,7 +834,7 @@
       </c>
       <c r="K7" s="5" t="inlineStr">
         <is>
-          <t>45 years x 3,108 counties x 12 months = 1,678,320 rows in a complete build.</t>
+          <t>A complete build is 45 years x 3,108 counties x 12 months = 1,678,320 rows.</t>
         </is>
       </c>
     </row>
@@ -875,7 +867,7 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Derived from the daily extraction date</t>
+          <t>Daily extraction date</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
@@ -885,7 +877,7 @@
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>Parsed from the daily `date` column; becomes the j() variable in the SECTION 1/2 `reshape wide`</t>
+          <t>j() variable in the SECTION 1/2 reshape wide</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
@@ -895,7 +887,7 @@
       </c>
       <c r="K8" s="5" t="inlineStr">
         <is>
-          <t>Every monthly measure below appears in main_data_county_year.dta as 12 columns, &lt;var&gt;_m1 ... &lt;var&gt;_m12. The _m suffix was a 9/5/26 call (Stata's own reshape produces a bare `mean_temp_c1`).</t>
+          <t>Every monthly measure below appears in main_data_county_year.dta as 12 columns, &lt;var&gt;_m1 ... &lt;var&gt;_m12.</t>
         </is>
       </c>
     </row>
@@ -928,7 +920,7 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd via 02a_extract_prism_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
+          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -938,17 +930,17 @@
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>count of daily rows in the geoid-year-month group (05)</t>
+          <t>Count of daily rows in the geoid-year-month group</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>No (collapsed to n_incomplete_months)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K9" s="5" t="inlineStr">
         <is>
-          <t>Compare against expected_days; a short month means days were missing from the extract, not that the county had fewer days.</t>
+          <t>Compare against expected_days: a short month means days were missing from the extract.</t>
         </is>
       </c>
     </row>
@@ -981,7 +973,7 @@
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd via 02a_extract_prism_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
+          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
@@ -991,17 +983,17 @@
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>05_aggregate_daily_to_monthly.py: sum of daily ppt within geoid-year-month (DatasetConfig sum-vs-mean lists)</t>
+          <t>05: sum of daily ppt within geoid-year-month</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>No (descriptives only)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr">
         <is>
-          <t>PRISM's own documentation notes its monthly grids are not a pure sum of the dailies (the monthly product uses more input stations), so this can differ slightly from PRISM's official monthly ppt grid. 06 computes the same quantity by a different route and 06b cross-checks the two.</t>
+          <t>PRISM's monthly grids are not a pure sum of its dailies (the monthly product uses more input stations), so this can differ slightly from PRISM's official monthly ppt grid.</t>
         </is>
       </c>
     </row>
@@ -1034,7 +1026,7 @@
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd via 02a_extract_prism_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
+          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
@@ -1044,12 +1036,12 @@
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>05_aggregate_daily_to_monthly.py: mean of daily tmean within geoid-year-month (DatasetConfig sum-vs-mean lists)</t>
+          <t>05: mean of daily tmean within geoid-year-month</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>No (descriptives only)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K11" s="5" t="inlineStr"/>
@@ -1083,7 +1075,7 @@
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd via 02a_extract_prism_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
+          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
@@ -1093,12 +1085,12 @@
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>05_aggregate_daily_to_monthly.py: mean of daily tmin within geoid-year-month (DatasetConfig sum-vs-mean lists)</t>
+          <t>05: mean of daily tmin within geoid-year-month</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>No (descriptives only)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr"/>
@@ -1132,7 +1124,7 @@
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd via 02a_extract_prism_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
+          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
@@ -1142,12 +1134,12 @@
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>05_aggregate_daily_to_monthly.py: mean of daily tmax within geoid-year-month (DatasetConfig sum-vs-mean lists)</t>
+          <t>05: mean of daily tmax within geoid-year-month</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>No (descriptives only)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K13" s="5" t="inlineStr"/>
@@ -1181,7 +1173,7 @@
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd via 02a_extract_prism_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
+          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
@@ -1191,17 +1183,17 @@
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>05_aggregate_daily_to_monthly.py: mean of daily tdmean within geoid-year-month (DatasetConfig sum-vs-mean lists)</t>
+          <t>05: mean of daily tdmean within geoid-year-month</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>No (descriptives only)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
-          <t>ERA5's dewpoint_c_mean is the closest counterpart but the two products compute dew point differently -- not like-for-like.</t>
+          <t>ERA5's dewpoint_c_mean is the closest counterpart, but the two products compute dew point differently -- not like-for-like.</t>
         </is>
       </c>
     </row>
@@ -1234,7 +1226,7 @@
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd via 02a_extract_prism_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
+          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
@@ -1244,12 +1236,12 @@
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>05_aggregate_daily_to_monthly.py: mean of daily vpdmin within geoid-year-month (DatasetConfig sum-vs-mean lists)</t>
+          <t>05: mean of daily vpdmin within geoid-year-month</t>
         </is>
       </c>
       <c r="J15" s="5" t="inlineStr">
         <is>
-          <t>No (descriptives only)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K15" s="5" t="inlineStr"/>
@@ -1283,7 +1275,7 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd via 02a_extract_prism_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
+          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
@@ -1293,12 +1285,12 @@
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t>05_aggregate_daily_to_monthly.py: mean of daily vpdmax within geoid-year-month (DatasetConfig sum-vs-mean lists)</t>
+          <t>05: mean of daily vpdmax within geoid-year-month</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>No (descriptives only)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K16" s="5" t="inlineStr"/>
@@ -1317,7 +1309,7 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>string (categorical, comma-joined)</t>
+          <t>string</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -1342,17 +1334,17 @@
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>Comma-joined sorted set of the daily rows' dataset_type</t>
+          <t>Comma-joined set of the daily rows' dataset_type</t>
         </is>
       </c>
       <c r="J17" s="5" t="inlineStr">
         <is>
-          <t>No (dropped in SECTION 1)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K17" s="5" t="inlineStr">
         <is>
-          <t>Flags county-months that mix vintages -- expected at the 2020/2021 boundary. Mixed months are printed by 05 rather than silently averaged. No ERA5 equivalent (ERA5-Land is a single reanalysis product).</t>
+          <t>Mixed-vintage months are expected at the 2020/2021 boundary. ERA5-Land has no equivalent (single reanalysis product).</t>
         </is>
       </c>
     </row>
@@ -1385,7 +1377,7 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Computed, not sourced (Python calendar.monthrange)</t>
+          <t>Computed (calendar.monthrange)</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
@@ -1400,7 +1392,7 @@
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>No (dropped in SECTION 1)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K18" s="5" t="inlineStr">
@@ -1418,7 +1410,7 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Flag: n_days != expected_days (partial daily coverage)</t>
+          <t>Flag: n_days does not match expected_days</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
@@ -1453,7 +1445,7 @@
       </c>
       <c r="J19" s="5" t="inlineStr">
         <is>
-          <t>No -- collapsed to n_incomplete_months in SECTION 1</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K19" s="5" t="inlineStr">
@@ -1476,7 +1468,7 @@
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>5-digit county FIPS (2-digit state + 3-digit county); the canonical merge key against every other RA's county-level panel</t>
+          <t>5-digit county FIPS (state + county); the merge key against every other county-level panel</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
@@ -1496,7 +1488,7 @@
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/ERA5/era5_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of ECMWF/ERA5_LAND/DAILY_AGGR via 04a_extract_era5_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/ERA5/extracted/county_daily_year)</t>
+          <t>dataRAW/ERA5/era5_county_daily_&lt;year&gt;.csv (GEE export of ECMWF/ERA5_LAND/DAILY_AGGR; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/ERA5/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr">
@@ -1506,17 +1498,17 @@
       </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
-          <t>Written by the GEE extraction; imported into Stata with stringcols(1 2 3) so leading zeros survive</t>
+          <t>Imported with stringcols(1 2 3) so leading zeros survive</t>
         </is>
       </c>
       <c r="J20" s="5" t="inlineStr">
         <is>
-          <t>No (only the five snow variables from 06 reach the merge)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K20" s="5" t="inlineStr">
         <is>
-          <t>Text, not numeric -- leading zeros are meaningful. Merge on geoid, never on county_name (names are not unique across states). County universe is TIGER/2018 everywhere in this pipeline. ERA5-Land is the robustness check against PRISM, not a co-equal weather source -- see project memory weather-pipeline-dataset-roles.</t>
+          <t>Text, not numeric. Merge on geoid, never on county_name. County universe is TIGER/2018 throughout. ERA5-Land is the robustness check against PRISM, not a co-equal source.</t>
         </is>
       </c>
     </row>
@@ -1549,7 +1541,7 @@
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>TIGER/2018/Counties (Earth Engine FeatureCollection), carried through the GEE extraction</t>
+          <t>TIGER/2018/Counties (Earth Engine FeatureCollection)</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
@@ -1559,19 +1551,15 @@
       </c>
       <c r="I21" s="5" t="inlineStr">
         <is>
-          <t>Carried through from the extraction; stringcols on import</t>
+          <t>Carried through from the extraction</t>
         </is>
       </c>
       <c r="J21" s="5" t="inlineStr">
         <is>
-          <t>No (only the five snow variables from 06 reach the merge)</t>
-        </is>
-      </c>
-      <c r="K21" s="5" t="inlineStr">
-        <is>
-          <t>CONUS scope is defined once, in gee_extract_utils.CONUS_STATE_FIPS, and imported by every extraction script.</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="n"/>
@@ -1602,7 +1590,7 @@
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>TIGER/2018/Counties (Earth Engine FeatureCollection), carried through the GEE extraction</t>
+          <t>TIGER/2018/Counties (Earth Engine FeatureCollection)</t>
         </is>
       </c>
       <c r="H22" s="5" t="inlineStr">
@@ -1612,19 +1600,15 @@
       </c>
       <c r="I22" s="5" t="inlineStr">
         <is>
-          <t>Carried through from the extraction; stringcols on import</t>
+          <t>Carried through from the extraction</t>
         </is>
       </c>
       <c r="J22" s="5" t="inlineStr">
         <is>
-          <t>No (only the five snow variables from 06 reach the merge)</t>
-        </is>
-      </c>
-      <c r="K22" s="5" t="inlineStr">
-        <is>
-          <t>Combine with state_fips for a nationally unique key, or just use geoid.</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="n"/>
@@ -1655,7 +1639,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>TIGER/2018/Counties (Earth Engine FeatureCollection), carried through the GEE extraction</t>
+          <t>TIGER/2018/Counties (Earth Engine FeatureCollection)</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -1670,12 +1654,12 @@
       </c>
       <c r="J23" s="5" t="inlineStr">
         <is>
-          <t>No (only the five snow variables from 06 reach the merge)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K23" s="5" t="inlineStr">
         <is>
-          <t>Reference/QA only -- not unique across states, so never a merge key.</t>
+          <t>Reference only -- not unique across states, so never a merge key.</t>
         </is>
       </c>
     </row>
@@ -1708,7 +1692,7 @@
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Derived from the daily extraction date</t>
+          <t>Daily extraction date</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr">
@@ -1718,7 +1702,7 @@
       </c>
       <c r="I24" s="5" t="inlineStr">
         <is>
-          <t>Parsed from the daily `date` column during aggregation</t>
+          <t>Parsed from the daily date column</t>
         </is>
       </c>
       <c r="J24" s="5" t="inlineStr">
@@ -1728,7 +1712,7 @@
       </c>
       <c r="K24" s="5" t="inlineStr">
         <is>
-          <t>45 years x 3,108 counties x 12 months = 1,678,320 rows in a complete build.</t>
+          <t>A complete build is 45 years x 3,108 counties x 12 months = 1,678,320 rows.</t>
         </is>
       </c>
     </row>
@@ -1761,7 +1745,7 @@
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>Derived from the daily extraction date</t>
+          <t>Daily extraction date</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr">
@@ -1771,7 +1755,7 @@
       </c>
       <c r="I25" s="5" t="inlineStr">
         <is>
-          <t>Parsed from the daily `date` column; becomes the j() variable in the SECTION 1/2 `reshape wide`</t>
+          <t>j() variable in the SECTION 1/2 reshape wide</t>
         </is>
       </c>
       <c r="J25" s="5" t="inlineStr">
@@ -1781,7 +1765,7 @@
       </c>
       <c r="K25" s="5" t="inlineStr">
         <is>
-          <t>Every monthly measure below appears in main_data_county_year.dta as 12 columns, &lt;var&gt;_m1 ... &lt;var&gt;_m12. The _m suffix was a 9/5/26 call (Stata's own reshape produces a bare `mean_temp_c1`).</t>
+          <t>Every monthly measure below appears in main_data_county_year.dta as 12 columns, &lt;var&gt;_m1 ... &lt;var&gt;_m12.</t>
         </is>
       </c>
     </row>
@@ -1814,7 +1798,7 @@
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/ERA5/era5_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of ECMWF/ERA5_LAND/DAILY_AGGR via 04a_extract_era5_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/ERA5/extracted/county_daily_year)</t>
+          <t>dataRAW/ERA5/era5_county_daily_&lt;year&gt;.csv (GEE export of ECMWF/ERA5_LAND/DAILY_AGGR; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/ERA5/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H26" s="5" t="inlineStr">
@@ -1824,17 +1808,17 @@
       </c>
       <c r="I26" s="5" t="inlineStr">
         <is>
-          <t>count of daily rows in the geoid-year-month group (05)</t>
+          <t>Count of daily rows in the geoid-year-month group</t>
         </is>
       </c>
       <c r="J26" s="5" t="inlineStr">
         <is>
-          <t>No (collapsed to n_incomplete_months)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K26" s="5" t="inlineStr">
         <is>
-          <t>Compare against expected_days; a short month means days were missing from the extract, not that the county had fewer days.</t>
+          <t>Compare against expected_days: a short month means days were missing from the extract.</t>
         </is>
       </c>
     </row>
@@ -1867,7 +1851,7 @@
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/ERA5/era5_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of ECMWF/ERA5_LAND/DAILY_AGGR via 04a_extract_era5_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/ERA5/extracted/county_daily_year)</t>
+          <t>dataRAW/ERA5/era5_county_daily_&lt;year&gt;.csv (GEE export of ECMWF/ERA5_LAND/DAILY_AGGR; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/ERA5/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr">
@@ -1877,17 +1861,17 @@
       </c>
       <c r="I27" s="5" t="inlineStr">
         <is>
-          <t>05_aggregate_daily_to_monthly.py: sum of daily precip_mm within geoid-year-month</t>
+          <t>05: sum of daily precip_mm within geoid-year-month</t>
         </is>
       </c>
       <c r="J27" s="5" t="inlineStr">
         <is>
-          <t>No (descriptives only)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K27" s="5" t="inlineStr">
         <is>
-          <t>Converted m-&gt;mm inline during extraction to match PRISM's convention; native ERA5-Land unit is metres.</t>
+          <t>Converted metres-&gt;mm during extraction to match PRISM's convention.</t>
         </is>
       </c>
     </row>
@@ -1920,7 +1904,7 @@
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/ERA5/era5_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of ECMWF/ERA5_LAND/DAILY_AGGR via 04a_extract_era5_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/ERA5/extracted/county_daily_year)</t>
+          <t>dataRAW/ERA5/era5_county_daily_&lt;year&gt;.csv (GEE export of ECMWF/ERA5_LAND/DAILY_AGGR; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/ERA5/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H28" s="5" t="inlineStr">
@@ -1930,17 +1914,17 @@
       </c>
       <c r="I28" s="5" t="inlineStr">
         <is>
-          <t>05_aggregate_daily_to_monthly.py: sum of daily snowfall_mm within geoid-year-month</t>
+          <t>05: sum of daily snowfall_mm within geoid-year-month</t>
         </is>
       </c>
       <c r="J28" s="5" t="inlineStr">
         <is>
-          <t>No (descriptives only)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K28" s="5" t="inlineStr">
         <is>
-          <t>PRISM has no equivalent -- ERA5-only.</t>
+          <t>ERA5-only; PRISM has no snow variable.</t>
         </is>
       </c>
     </row>
@@ -1973,7 +1957,7 @@
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/ERA5/era5_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of ECMWF/ERA5_LAND/DAILY_AGGR via 04a_extract_era5_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/ERA5/extracted/county_daily_year)</t>
+          <t>dataRAW/ERA5/era5_county_daily_&lt;year&gt;.csv (GEE export of ECMWF/ERA5_LAND/DAILY_AGGR; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/ERA5/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr">
@@ -1983,12 +1967,12 @@
       </c>
       <c r="I29" s="5" t="inlineStr">
         <is>
-          <t>05_aggregate_daily_to_monthly.py: mean of daily tmean_c within geoid-year-month</t>
+          <t>05: mean of daily tmean_c within geoid-year-month</t>
         </is>
       </c>
       <c r="J29" s="5" t="inlineStr">
         <is>
-          <t>No (descriptives only)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K29" s="5" t="inlineStr">
@@ -2026,7 +2010,7 @@
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/ERA5/era5_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of ECMWF/ERA5_LAND/DAILY_AGGR via 04a_extract_era5_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/ERA5/extracted/county_daily_year)</t>
+          <t>dataRAW/ERA5/era5_county_daily_&lt;year&gt;.csv (GEE export of ECMWF/ERA5_LAND/DAILY_AGGR; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/ERA5/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H30" s="5" t="inlineStr">
@@ -2036,17 +2020,17 @@
       </c>
       <c r="I30" s="5" t="inlineStr">
         <is>
-          <t>05_aggregate_daily_to_monthly.py: mean of daily tmin_c within geoid-year-month</t>
+          <t>05: mean of daily tmin_c within geoid-year-month</t>
         </is>
       </c>
       <c r="J30" s="5" t="inlineStr">
         <is>
-          <t>No (descriptives only)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K30" s="5" t="inlineStr">
         <is>
-          <t>Added after the 03a small-scale test. Duplicates PRISM's tmin_mean by design: ERA5 needs its own tmin/tmax to serve as a robustness check against PRISM.</t>
+          <t>Duplicates PRISM's tmin_mean by design -- ERA5 needs its own tmin/tmax to serve as a robustness check. The base names collide, so do not merge both into one panel unrenamed.</t>
         </is>
       </c>
     </row>
@@ -2079,7 +2063,7 @@
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/ERA5/era5_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of ECMWF/ERA5_LAND/DAILY_AGGR via 04a_extract_era5_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/ERA5/extracted/county_daily_year)</t>
+          <t>dataRAW/ERA5/era5_county_daily_&lt;year&gt;.csv (GEE export of ECMWF/ERA5_LAND/DAILY_AGGR; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/ERA5/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr">
@@ -2089,17 +2073,17 @@
       </c>
       <c r="I31" s="5" t="inlineStr">
         <is>
-          <t>05_aggregate_daily_to_monthly.py: mean of daily tmax_c within geoid-year-month</t>
+          <t>05: mean of daily tmax_c within geoid-year-month</t>
         </is>
       </c>
       <c r="J31" s="5" t="inlineStr">
         <is>
-          <t>No (descriptives only)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K31" s="5" t="inlineStr">
         <is>
-          <t>Same reasoning as tmin_c_mean.</t>
+          <t>Same as tmin_c_mean.</t>
         </is>
       </c>
     </row>
@@ -2132,7 +2116,7 @@
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/ERA5/era5_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of ECMWF/ERA5_LAND/DAILY_AGGR via 04a_extract_era5_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/ERA5/extracted/county_daily_year)</t>
+          <t>dataRAW/ERA5/era5_county_daily_&lt;year&gt;.csv (GEE export of ECMWF/ERA5_LAND/DAILY_AGGR; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/ERA5/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H32" s="5" t="inlineStr">
@@ -2142,17 +2126,17 @@
       </c>
       <c r="I32" s="5" t="inlineStr">
         <is>
-          <t>05_aggregate_daily_to_monthly.py: mean of daily dewpoint_c within geoid-year-month</t>
+          <t>05: mean of daily dewpoint_c within geoid-year-month</t>
         </is>
       </c>
       <c r="J32" s="5" t="inlineStr">
         <is>
-          <t>No (descriptives only)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K32" s="5" t="inlineStr">
         <is>
-          <t>PRISM's tdmean_mean is the closest counterpart, but the two are computed differently.</t>
+          <t>PRISM's tdmean_mean is the closest counterpart, computed differently.</t>
         </is>
       </c>
     </row>
@@ -2185,7 +2169,7 @@
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/ERA5/era5_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of ECMWF/ERA5_LAND/DAILY_AGGR via 04a_extract_era5_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/ERA5/extracted/county_daily_year)</t>
+          <t>dataRAW/ERA5/era5_county_daily_&lt;year&gt;.csv (GEE export of ECMWF/ERA5_LAND/DAILY_AGGR; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/ERA5/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H33" s="5" t="inlineStr">
@@ -2195,17 +2179,17 @@
       </c>
       <c r="I33" s="5" t="inlineStr">
         <is>
-          <t>05_aggregate_daily_to_monthly.py: mean of daily skin_temp_c within geoid-year-month</t>
+          <t>05: mean of daily skin_temp_c within geoid-year-month</t>
         </is>
       </c>
       <c r="J33" s="5" t="inlineStr">
         <is>
-          <t>No (descriptives only)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K33" s="5" t="inlineStr">
         <is>
-          <t>Land surface, not 2m air temperature. PRISM has no equivalent.</t>
+          <t>Land surface, not 2m air temperature. No PRISM equivalent.</t>
         </is>
       </c>
     </row>
@@ -2238,7 +2222,7 @@
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/ERA5/era5_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of ECMWF/ERA5_LAND/DAILY_AGGR via 04a_extract_era5_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/ERA5/extracted/county_daily_year)</t>
+          <t>dataRAW/ERA5/era5_county_daily_&lt;year&gt;.csv (GEE export of ECMWF/ERA5_LAND/DAILY_AGGR; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/ERA5/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H34" s="5" t="inlineStr">
@@ -2248,17 +2232,17 @@
       </c>
       <c r="I34" s="5" t="inlineStr">
         <is>
-          <t>05_aggregate_daily_to_monthly.py: mean of daily wind speed within geoid-year-month</t>
+          <t>05: mean of daily wind speed within geoid-year-month</t>
         </is>
       </c>
       <c r="J34" s="5" t="inlineStr">
         <is>
-          <t>No (descriptives only)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K34" s="5" t="inlineStr">
         <is>
-          <t>ERA5-Land has no wind-speed band; computed as sqrt(u^2+v^2) from the u/v components during extraction, from the DAILY MEAN components (not the mean of hourly speeds). PRISM has no wind variable.</t>
+          <t>ERA5-Land has no wind-speed band: computed as sqrt(u^2+v^2) from the daily mean u/v components, not the mean of hourly speeds. No PRISM equivalent.</t>
         </is>
       </c>
     </row>
@@ -2286,12 +2270,12 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>continuous, metres (native ERA5-Land unit, not converted)</t>
+          <t>continuous, metres (native ERA5-Land unit)</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/ERA5/era5_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of ECMWF/ERA5_LAND/DAILY_AGGR via 04a_extract_era5_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/ERA5/extracted/county_daily_year)</t>
+          <t>dataRAW/ERA5/era5_county_daily_&lt;year&gt;.csv (GEE export of ECMWF/ERA5_LAND/DAILY_AGGR; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/ERA5/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H35" s="5" t="inlineStr">
@@ -2301,17 +2285,17 @@
       </c>
       <c r="I35" s="5" t="inlineStr">
         <is>
-          <t>05_aggregate_daily_to_monthly.py: mean of daily snow_depth within geoid-year-month</t>
+          <t>05: mean of daily snow_depth within geoid-year-month</t>
         </is>
       </c>
       <c r="J35" s="5" t="inlineStr">
         <is>
-          <t>No (descriptives only)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K35" s="5" t="inlineStr">
         <is>
-          <t>Averaged, not summed: snow depth is a stock, not a flux. This is the snow_depth band (thickness on the ground), NOT snow_depth_water_equivalent. PRISM has no equivalent.</t>
+          <t>Averaged, not summed -- snow depth is a stock. This is the snow_depth band (thickness on the ground), not snow_depth_water_equivalent.</t>
         </is>
       </c>
     </row>
@@ -2339,12 +2323,12 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>continuous, Pa (native ERA5-Land unit, not converted)</t>
+          <t>continuous, Pa (native ERA5-Land unit)</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/ERA5/era5_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of ECMWF/ERA5_LAND/DAILY_AGGR via 04a_extract_era5_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/ERA5/extracted/county_daily_year)</t>
+          <t>dataRAW/ERA5/era5_county_daily_&lt;year&gt;.csv (GEE export of ECMWF/ERA5_LAND/DAILY_AGGR; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/ERA5/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H36" s="5" t="inlineStr">
@@ -2354,17 +2338,17 @@
       </c>
       <c r="I36" s="5" t="inlineStr">
         <is>
-          <t>05_aggregate_daily_to_monthly.py: mean of daily surface_pressure within geoid-year-month</t>
+          <t>05: mean of daily surface_pressure within geoid-year-month</t>
         </is>
       </c>
       <c r="J36" s="5" t="inlineStr">
         <is>
-          <t>No (descriptives only)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K36" s="5" t="inlineStr">
         <is>
-          <t>PRISM has no equivalent.</t>
+          <t>No PRISM equivalent.</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2410,7 @@
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>Flag: n_days != expected_days</t>
+          <t>Flag: n_days does not match expected_days</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
@@ -2484,7 +2468,7 @@
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>5-digit county FIPS (2-digit state + 3-digit county); the canonical merge key against every other RA's county-level panel</t>
+          <t>5-digit county FIPS (state + county); the merge key against every other county-level panel</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
@@ -2504,7 +2488,7 @@
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd via 02a_extract_prism_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
+          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H39" s="5" t="inlineStr">
@@ -2514,7 +2498,7 @@
       </c>
       <c r="I39" s="5" t="inlineStr">
         <is>
-          <t>Written by the GEE extraction; imported into Stata with stringcols(1 2 3) so leading zeros survive</t>
+          <t>Imported with stringcols(1 2 3) so leading zeros survive</t>
         </is>
       </c>
       <c r="J39" s="5" t="inlineStr">
@@ -2524,7 +2508,7 @@
       </c>
       <c r="K39" s="5" t="inlineStr">
         <is>
-          <t>Text, not numeric -- leading zeros are meaningful. Merge on geoid, never on county_name (names are not unique across states). County universe is TIGER/2018 everywhere in this pipeline. THIS is the file SECTION 1 of build_main_data_county_year.do reads -- it, not prism_county_month.csv, is the merge input and the master spine of main_data_county_year.dta.</t>
+          <t>Text, not numeric. Merge on geoid, never on county_name. County universe is TIGER/2018 throughout. This is the file SECTION 1 reads; it is the master spine of main_data_county_year.dta.</t>
         </is>
       </c>
     </row>
@@ -2557,7 +2541,7 @@
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>TIGER/2018/Counties (Earth Engine FeatureCollection), carried through the GEE extraction</t>
+          <t>TIGER/2018/Counties (Earth Engine FeatureCollection)</t>
         </is>
       </c>
       <c r="H40" s="5" t="inlineStr">
@@ -2567,7 +2551,7 @@
       </c>
       <c r="I40" s="5" t="inlineStr">
         <is>
-          <t>Carried through from the extraction; stringcols on import</t>
+          <t>Carried through from the extraction</t>
         </is>
       </c>
       <c r="J40" s="5" t="inlineStr">
@@ -2575,11 +2559,7 @@
           <t>Yes (panel key)</t>
         </is>
       </c>
-      <c r="K40" s="5" t="inlineStr">
-        <is>
-          <t>CONUS scope is defined once, in gee_extract_utils.CONUS_STATE_FIPS, and imported by every extraction script.</t>
-        </is>
-      </c>
+      <c r="K40" s="5" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="5" t="n"/>
@@ -2610,7 +2590,7 @@
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>TIGER/2018/Counties (Earth Engine FeatureCollection), carried through the GEE extraction</t>
+          <t>TIGER/2018/Counties (Earth Engine FeatureCollection)</t>
         </is>
       </c>
       <c r="H41" s="5" t="inlineStr">
@@ -2620,7 +2600,7 @@
       </c>
       <c r="I41" s="5" t="inlineStr">
         <is>
-          <t>Carried through from the extraction; stringcols on import</t>
+          <t>Carried through from the extraction</t>
         </is>
       </c>
       <c r="J41" s="5" t="inlineStr">
@@ -2628,11 +2608,7 @@
           <t>Yes (panel key)</t>
         </is>
       </c>
-      <c r="K41" s="5" t="inlineStr">
-        <is>
-          <t>Combine with state_fips for a nationally unique key, or just use geoid.</t>
-        </is>
-      </c>
+      <c r="K41" s="5" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="5" t="n"/>
@@ -2663,7 +2639,7 @@
       </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>TIGER/2018/Counties (Earth Engine FeatureCollection), carried through the GEE extraction</t>
+          <t>TIGER/2018/Counties (Earth Engine FeatureCollection)</t>
         </is>
       </c>
       <c r="H42" s="5" t="inlineStr">
@@ -2683,7 +2659,7 @@
       </c>
       <c r="K42" s="5" t="inlineStr">
         <is>
-          <t>Reference/QA only -- not unique across states, so never a merge key.</t>
+          <t>Reference only -- not unique across states, so never a merge key.</t>
         </is>
       </c>
     </row>
@@ -2716,7 +2692,7 @@
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>Derived from the daily extraction date</t>
+          <t>Daily extraction date</t>
         </is>
       </c>
       <c r="H43" s="5" t="inlineStr">
@@ -2726,7 +2702,7 @@
       </c>
       <c r="I43" s="5" t="inlineStr">
         <is>
-          <t>Parsed from the daily `date` column during aggregation</t>
+          <t>Parsed from the daily date column</t>
         </is>
       </c>
       <c r="J43" s="5" t="inlineStr">
@@ -2736,7 +2712,7 @@
       </c>
       <c r="K43" s="5" t="inlineStr">
         <is>
-          <t>45 years x 3,108 counties x 12 months = 1,678,320 rows in a complete build.</t>
+          <t>A complete build is 45 years x 3,108 counties x 12 months = 1,678,320 rows.</t>
         </is>
       </c>
     </row>
@@ -2769,7 +2745,7 @@
       </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>Derived from the daily extraction date</t>
+          <t>Daily extraction date</t>
         </is>
       </c>
       <c r="H44" s="5" t="inlineStr">
@@ -2779,7 +2755,7 @@
       </c>
       <c r="I44" s="5" t="inlineStr">
         <is>
-          <t>Parsed from the daily `date` column; becomes the j() variable in the SECTION 1/2 `reshape wide`</t>
+          <t>j() variable in the SECTION 1/2 reshape wide</t>
         </is>
       </c>
       <c r="J44" s="5" t="inlineStr">
@@ -2789,7 +2765,7 @@
       </c>
       <c r="K44" s="5" t="inlineStr">
         <is>
-          <t>Every monthly measure below appears in main_data_county_year.dta as 12 columns, &lt;var&gt;_m1 ... &lt;var&gt;_m12. The _m suffix was a 9/5/26 call (Stata's own reshape produces a bare `mean_temp_c1`).</t>
+          <t>Every monthly measure below appears in main_data_county_year.dta as 12 columns, &lt;var&gt;_m1 ... &lt;var&gt;_m12.</t>
         </is>
       </c>
     </row>
@@ -2822,7 +2798,7 @@
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd via 02a_extract_prism_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
+          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H45" s="5" t="inlineStr">
@@ -2832,7 +2808,7 @@
       </c>
       <c r="I45" s="5" t="inlineStr">
         <is>
-          <t>count of daily rows in the geoid-year-month group (06)</t>
+          <t>Count of daily rows in the geoid-year-month group</t>
         </is>
       </c>
       <c r="J45" s="5" t="inlineStr">
@@ -2842,7 +2818,7 @@
       </c>
       <c r="K45" s="5" t="inlineStr">
         <is>
-          <t>Compare against expected_days; a short month means days were missing from the extract, not that the county had fewer days.</t>
+          <t>Compare against expected_days: a short month means days were missing from the extract.</t>
         </is>
       </c>
     </row>
@@ -2875,7 +2851,7 @@
       </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd via 02a_extract_prism_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
+          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H46" s="5" t="inlineStr">
@@ -2885,17 +2861,17 @@
       </c>
       <c r="I46" s="5" t="inlineStr">
         <is>
-          <t>06_build_derived_weather_vars.py: sum of daily ppt, grouped by geoid-year-month. Stata SECTION 1 then reshapes wide by month and renames to _m1.._m12.</t>
+          <t>06: sum of daily ppt, grouped by geoid-year-month; SECTION 1 then reshapes wide by month and renames to _m1.._m12</t>
         </is>
       </c>
       <c r="J46" s="5" t="inlineStr">
         <is>
-          <t>Yes, reshaped wide as &lt;var&gt;_m1 .. &lt;var&gt;_m12 (SECTION 1)</t>
+          <t>Yes, as &lt;var&gt;_m1 .. &lt;var&gt;_m12 (SECTION 1)</t>
         </is>
       </c>
       <c r="K46" s="5" t="inlineStr">
         <is>
-          <t>Named after each dataset's own precip column exactly as 05 does, so the two files cross-check column for column -- that is what 06b_validate_ppt_total.py compares. pandas sum() skips NaN, so a month with missing days is understated rather than missing. Feeds the annual precipitation quintile control downstream.</t>
+          <t>Computed from the dailies independently of 05, which produces the same quantity by a different route; 06b compares the two. A month with missing days is understated, not missing.</t>
         </is>
       </c>
     </row>
@@ -2928,7 +2904,7 @@
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd via 02a_extract_prism_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
+          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H47" s="5" t="inlineStr">
@@ -2938,17 +2914,17 @@
       </c>
       <c r="I47" s="5" t="inlineStr">
         <is>
-          <t>06_build_derived_weather_vars.py: count of daily tmin &lt;= -17.7778C, grouped by geoid-year-month. Stata SECTION 1 then reshapes wide by month and renames to _m1.._m12.</t>
+          <t>06: count of daily tmin &lt;= -17.7778C, grouped by geoid-year-month; SECTION 1 then reshapes wide by month and renames to _m1.._m12</t>
         </is>
       </c>
       <c r="J47" s="5" t="inlineStr">
         <is>
-          <t>Yes, reshaped wide as &lt;var&gt;_m1 .. &lt;var&gt;_m12 (SECTION 1)</t>
+          <t>Yes, as &lt;var&gt;_m1 .. &lt;var&gt;_m12 (SECTION 1)</t>
         </is>
       </c>
       <c r="K47" s="5" t="inlineStr">
         <is>
-          <t>INCLUSIVE (&lt;=) deliberately: it is the cold-stress component of the Kohn (1975) winter severity index, defined on 'a minimum temperature of 0F or below'. Changed from strict &lt; on 09/08/2026 -- moves zero county-days in the 1981 and 2025 extracts, so a definitional correction, not a numbers change. This is the deer metabolic-stress / lagged population-prediction threshold, NOT the road-conditions one.</t>
+          <t>INCLUSIVE (&lt;=), following Kohn (1975)'s 'a minimum temperature of 0F or below'. This is the deer metabolic-stress threshold and the WSI's cold component -- NOT the road-conditions variable.</t>
         </is>
       </c>
     </row>
@@ -2981,7 +2957,7 @@
       </c>
       <c r="G48" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd via 02a_extract_prism_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
+          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H48" s="5" t="inlineStr">
@@ -2991,17 +2967,17 @@
       </c>
       <c r="I48" s="5" t="inlineStr">
         <is>
-          <t>06_build_derived_weather_vars.py: count of daily tmin &lt; 0C, grouped by geoid-year-month. Stata SECTION 1 then reshapes wide by month and renames to _m1.._m12.</t>
+          <t>06: count of daily tmin &lt; 0C, grouped by geoid-year-month; SECTION 1 then reshapes wide by month and renames to _m1.._m12</t>
         </is>
       </c>
       <c r="J48" s="5" t="inlineStr">
         <is>
-          <t>Yes, reshaped wide as &lt;var&gt;_m1 .. &lt;var&gt;_m12 (SECTION 1)</t>
+          <t>Yes, as &lt;var&gt;_m1 .. &lt;var&gt;_m12 (SECTION 1)</t>
         </is>
       </c>
       <c r="K48" s="5" t="inlineStr">
         <is>
-          <t>STRICT (&lt;) deliberately -- the standard definition of a below-freezing day, and not part of the WSI. Split from days_extremely_cold at the 08/14/2026 team meeting: this is the contemporaneous icy-road covariate, the other is the deer-population instrument. Do not conflate the two.</t>
+          <t>STRICT (&lt;) -- the standard below-freezing day, not part of the WSI. This is the contemporaneous icy-road covariate. Do not conflate with days_extremely_cold.</t>
         </is>
       </c>
     </row>
@@ -3034,7 +3010,7 @@
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd via 02a_extract_prism_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
+          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H49" s="5" t="inlineStr">
@@ -3044,12 +3020,12 @@
       </c>
       <c r="I49" s="5" t="inlineStr">
         <is>
-          <t>06_build_derived_weather_vars.py: count of daily (tmin &lt; 0C) &amp; (tmax &gt; 0C), grouped by geoid-year-month. Stata SECTION 1 then reshapes wide by month and renames to _m1.._m12.</t>
+          <t>06: count of daily (tmin &lt; 0C) &amp; (tmax &gt; 0C), grouped by geoid-year-month; SECTION 1 then reshapes wide by month and renames to _m1.._m12</t>
         </is>
       </c>
       <c r="J49" s="5" t="inlineStr">
         <is>
-          <t>Yes, reshaped wide as &lt;var&gt;_m1 .. &lt;var&gt;_m12 (SECTION 1)</t>
+          <t>Yes, as &lt;var&gt;_m1 .. &lt;var&gt;_m12 (SECTION 1)</t>
         </is>
       </c>
       <c r="K49" s="5" t="inlineStr"/>
@@ -3083,7 +3059,7 @@
       </c>
       <c r="G50" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd via 02a_extract_prism_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
+          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H50" s="5" t="inlineStr">
@@ -3093,17 +3069,17 @@
       </c>
       <c r="I50" s="5" t="inlineStr">
         <is>
-          <t>06_build_derived_weather_vars.py: count of daily ppt &gt; 10mm, grouped by geoid-year-month. Stata SECTION 1 then reshapes wide by month and renames to _m1.._m12.</t>
+          <t>06: count of daily ppt &gt; 10mm, grouped by geoid-year-month; SECTION 1 then reshapes wide by month and renames to _m1.._m12</t>
         </is>
       </c>
       <c r="J50" s="5" t="inlineStr">
         <is>
-          <t>Yes, reshaped wide as &lt;var&gt;_m1 .. &lt;var&gt;_m12 (SECTION 1)</t>
+          <t>Yes, as &lt;var&gt;_m1 .. &lt;var&gt;_m12 (SECTION 1)</t>
         </is>
       </c>
       <c r="K50" s="5" t="inlineStr">
         <is>
-          <t>Threshold is PRECIP_THRESHOLD_MM in 06; 10mm is the task doc's example value. Changing the constant changes the column name too.</t>
+          <t>Threshold is PRECIP_THRESHOLD_MM in 06; changing it changes the column name.</t>
         </is>
       </c>
     </row>
@@ -3136,7 +3112,7 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd via 02a_extract_prism_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
+          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">
@@ -3146,17 +3122,17 @@
       </c>
       <c r="I51" s="5" t="inlineStr">
         <is>
-          <t>06_build_derived_weather_vars.py: sum over days of max(18.33 - tmean, 0), grouped by geoid-year-month. Stata SECTION 1 then reshapes wide by month and renames to _m1.._m12.</t>
+          <t>06: sum over days of max(18.33 - tmean, 0), grouped by geoid-year-month; SECTION 1 then reshapes wide by month and renames to _m1.._m12</t>
         </is>
       </c>
       <c r="J51" s="5" t="inlineStr">
         <is>
-          <t>Yes, reshaped wide as &lt;var&gt;_m1 .. &lt;var&gt;_m12 (SECTION 1)</t>
+          <t>Yes, as &lt;var&gt;_m1 .. &lt;var&gt;_m12 (SECTION 1)</t>
         </is>
       </c>
       <c r="K51" s="5" t="inlineStr">
         <is>
-          <t>Base 65F is the standard US/NOAA convention, converted to C to match the datasets' native units.</t>
+          <t>Base 65F is the standard NOAA convention, converted to C.</t>
         </is>
       </c>
     </row>
@@ -3189,7 +3165,7 @@
       </c>
       <c r="G52" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd via 02a_extract_prism_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
+          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H52" s="5" t="inlineStr">
@@ -3199,12 +3175,12 @@
       </c>
       <c r="I52" s="5" t="inlineStr">
         <is>
-          <t>06_build_derived_weather_vars.py: sum over days of max(tmean - 18.33, 0), grouped by geoid-year-month. Stata SECTION 1 then reshapes wide by month and renames to _m1.._m12.</t>
+          <t>06: sum over days of max(tmean - 18.33, 0), grouped by geoid-year-month; SECTION 1 then reshapes wide by month and renames to _m1.._m12</t>
         </is>
       </c>
       <c r="J52" s="5" t="inlineStr">
         <is>
-          <t>Yes, reshaped wide as &lt;var&gt;_m1 .. &lt;var&gt;_m12 (SECTION 1)</t>
+          <t>Yes, as &lt;var&gt;_m1 .. &lt;var&gt;_m12 (SECTION 1)</t>
         </is>
       </c>
       <c r="K52" s="5" t="inlineStr"/>
@@ -3238,7 +3214,7 @@
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd via 02a_extract_prism_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
+          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H53" s="5" t="inlineStr">
@@ -3248,17 +3224,17 @@
       </c>
       <c r="I53" s="5" t="inlineStr">
         <is>
-          <t>06_build_derived_weather_vars.py: mean of daily tmean, grouped by geoid-year-month. Stata SECTION 1 then reshapes wide by month and renames to _m1.._m12.</t>
+          <t>06: mean of daily tmean, grouped by geoid-year-month; SECTION 1 then reshapes wide by month and renames to _m1.._m12</t>
         </is>
       </c>
       <c r="J53" s="5" t="inlineStr">
         <is>
-          <t>Yes, reshaped wide as &lt;var&gt;_m1 .. &lt;var&gt;_m12 (SECTION 1)</t>
+          <t>Yes, as &lt;var&gt;_m1 .. &lt;var&gt;_m12 (SECTION 1)</t>
         </is>
       </c>
       <c r="K53" s="5" t="inlineStr">
         <is>
-          <t>Computed from the daily extracts independently of 05, so it can be cross-checked against 05's tmean_mean. mean_temp_c_m12/_m1/_m2 are what SECTION 7 averages into mean_winter_temp.</t>
+          <t>mean_temp_c_m12/_m1/_m2 are what SECTION 7 averages into mean_winter_temp.</t>
         </is>
       </c>
     </row>
@@ -3291,7 +3267,7 @@
       </c>
       <c r="G54" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd via 02a_extract_prism_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
+          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H54" s="5" t="inlineStr">
@@ -3301,17 +3277,17 @@
       </c>
       <c r="I54" s="5" t="inlineStr">
         <is>
-          <t>06_build_derived_weather_vars.py: sample variance (ddof=1) of daily tmean, grouped by geoid-year-month. Stata SECTION 1 then reshapes wide by month and renames to _m1.._m12.</t>
+          <t>06: sample variance (ddof=1) of daily tmean, grouped by geoid-year-month; SECTION 1 then reshapes wide by month and renames to _m1.._m12</t>
         </is>
       </c>
       <c r="J54" s="5" t="inlineStr">
         <is>
-          <t>Yes, reshaped wide as &lt;var&gt;_m1 .. &lt;var&gt;_m12 (SECTION 1)</t>
+          <t>Yes, as &lt;var&gt;_m1 .. &lt;var&gt;_m12 (SECTION 1)</t>
         </is>
       </c>
       <c r="K54" s="5" t="inlineStr">
         <is>
-          <t>Sample variance, pandas default ddof=1 -- not the population variance.</t>
+          <t>Sample variance, not population variance.</t>
         </is>
       </c>
     </row>
@@ -3344,7 +3320,7 @@
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd via 02a_extract_prism_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
+          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H55" s="5" t="inlineStr">
@@ -3354,12 +3330,12 @@
       </c>
       <c r="I55" s="5" t="inlineStr">
         <is>
-          <t>06_build_derived_weather_vars.py: sample variance (ddof=1) of daily tmin, grouped by geoid-year-month. Stata SECTION 1 then reshapes wide by month and renames to _m1.._m12.</t>
+          <t>06: sample variance (ddof=1) of daily tmin, grouped by geoid-year-month; SECTION 1 then reshapes wide by month and renames to _m1.._m12</t>
         </is>
       </c>
       <c r="J55" s="5" t="inlineStr">
         <is>
-          <t>Yes, reshaped wide as &lt;var&gt;_m1 .. &lt;var&gt;_m12 (SECTION 1)</t>
+          <t>Yes, as &lt;var&gt;_m1 .. &lt;var&gt;_m12 (SECTION 1)</t>
         </is>
       </c>
       <c r="K55" s="5" t="inlineStr"/>
@@ -3393,7 +3369,7 @@
       </c>
       <c r="G56" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd via 02a_extract_prism_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
+          <t>dataRAW/PRISM/prism_county_daily_&lt;year&gt;.csv (GEE export of OREGONSTATE/PRISM/ANd; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/PRISM/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H56" s="5" t="inlineStr">
@@ -3403,12 +3379,12 @@
       </c>
       <c r="I56" s="5" t="inlineStr">
         <is>
-          <t>06_build_derived_weather_vars.py: sample variance (ddof=1) of daily tmax, grouped by geoid-year-month. Stata SECTION 1 then reshapes wide by month and renames to _m1.._m12.</t>
+          <t>06: sample variance (ddof=1) of daily tmax, grouped by geoid-year-month; SECTION 1 then reshapes wide by month and renames to _m1.._m12</t>
         </is>
       </c>
       <c r="J56" s="5" t="inlineStr">
         <is>
-          <t>Yes, reshaped wide as &lt;var&gt;_m1 .. &lt;var&gt;_m12 (SECTION 1)</t>
+          <t>Yes, as &lt;var&gt;_m1 .. &lt;var&gt;_m12 (SECTION 1)</t>
         </is>
       </c>
       <c r="K56" s="5" t="inlineStr"/>
@@ -3452,7 +3428,7 @@
       </c>
       <c r="I57" s="5" t="inlineStr">
         <is>
-          <t>Dropped in SECTION 1 before the reshape</t>
+          <t>Dropped in SECTION 1</t>
         </is>
       </c>
       <c r="J57" s="5" t="inlineStr">
@@ -3524,7 +3500,7 @@
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Flag: n_days != expected_days</t>
+          <t>Flag: n_days does not match expected_days</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
@@ -3559,12 +3535,12 @@
       </c>
       <c r="J59" s="5" t="inlineStr">
         <is>
-          <t>Indirectly -- as n_incomplete_months</t>
+          <t>Indirectly, as n_incomplete_months</t>
         </is>
       </c>
       <c r="K59" s="5" t="inlineStr">
         <is>
-          <t>Collapsed to one county-YEAR count rather than reshaped wide: a monthly True/False is a QA note, not an analysis variable.</t>
+          <t>Collapsed to one county-year count rather than reshaped wide.</t>
         </is>
       </c>
     </row>
@@ -3582,7 +3558,7 @@
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>5-digit county FIPS (2-digit state + 3-digit county); the canonical merge key against every other RA's county-level panel</t>
+          <t>5-digit county FIPS (state + county); the merge key against every other county-level panel</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
@@ -3602,7 +3578,7 @@
       </c>
       <c r="G60" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/ERA5/era5_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of ECMWF/ERA5_LAND/DAILY_AGGR via 04a_extract_era5_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/ERA5/extracted/county_daily_year)</t>
+          <t>dataRAW/ERA5/era5_county_daily_&lt;year&gt;.csv (GEE export of ECMWF/ERA5_LAND/DAILY_AGGR; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/ERA5/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H60" s="5" t="inlineStr">
@@ -3612,7 +3588,7 @@
       </c>
       <c r="I60" s="5" t="inlineStr">
         <is>
-          <t>Written by the GEE extraction; imported into Stata with stringcols(1 2 3) so leading zeros survive</t>
+          <t>Imported with stringcols(1 2 3) so leading zeros survive</t>
         </is>
       </c>
       <c r="J60" s="5" t="inlineStr">
@@ -3622,7 +3598,7 @@
       </c>
       <c r="K60" s="5" t="inlineStr">
         <is>
-          <t>Text, not numeric -- leading zeros are meaningful. Merge on geoid, never on county_name (names are not unique across states). County universe is TIGER/2018 everywhere in this pipeline. SECTION 2 keeps ONLY mean_snow_depth, total_snowfall_mm and the three days_snow_depth_* columns from this file; the temperature/precip columns are PRISM's job. The five are merged 1:1 on geoid year.</t>
+          <t>Text, not numeric. Merge on geoid, never on county_name. County universe is TIGER/2018 throughout. SECTION 2 keeps only mean_snow_depth, total_snowfall_mm and the three days_snow_depth_* columns, merged 1:1 on geoid year.</t>
         </is>
       </c>
     </row>
@@ -3655,7 +3631,7 @@
       </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
-          <t>TIGER/2018/Counties (Earth Engine FeatureCollection), carried through the GEE extraction</t>
+          <t>TIGER/2018/Counties (Earth Engine FeatureCollection)</t>
         </is>
       </c>
       <c r="H61" s="5" t="inlineStr">
@@ -3665,7 +3641,7 @@
       </c>
       <c r="I61" s="5" t="inlineStr">
         <is>
-          <t>Carried through from the extraction; stringcols on import</t>
+          <t>Carried through from the extraction</t>
         </is>
       </c>
       <c r="J61" s="5" t="inlineStr">
@@ -3673,11 +3649,7 @@
           <t>Snow variables only</t>
         </is>
       </c>
-      <c r="K61" s="5" t="inlineStr">
-        <is>
-          <t>CONUS scope is defined once, in gee_extract_utils.CONUS_STATE_FIPS, and imported by every extraction script.</t>
-        </is>
-      </c>
+      <c r="K61" s="5" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="5" t="n"/>
@@ -3708,7 +3680,7 @@
       </c>
       <c r="G62" s="5" t="inlineStr">
         <is>
-          <t>TIGER/2018/Counties (Earth Engine FeatureCollection), carried through the GEE extraction</t>
+          <t>TIGER/2018/Counties (Earth Engine FeatureCollection)</t>
         </is>
       </c>
       <c r="H62" s="5" t="inlineStr">
@@ -3718,7 +3690,7 @@
       </c>
       <c r="I62" s="5" t="inlineStr">
         <is>
-          <t>Carried through from the extraction; stringcols on import</t>
+          <t>Carried through from the extraction</t>
         </is>
       </c>
       <c r="J62" s="5" t="inlineStr">
@@ -3726,11 +3698,7 @@
           <t>Snow variables only</t>
         </is>
       </c>
-      <c r="K62" s="5" t="inlineStr">
-        <is>
-          <t>Combine with state_fips for a nationally unique key, or just use geoid.</t>
-        </is>
-      </c>
+      <c r="K62" s="5" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="5" t="n"/>
@@ -3761,7 +3729,7 @@
       </c>
       <c r="G63" s="5" t="inlineStr">
         <is>
-          <t>TIGER/2018/Counties (Earth Engine FeatureCollection), carried through the GEE extraction</t>
+          <t>TIGER/2018/Counties (Earth Engine FeatureCollection)</t>
         </is>
       </c>
       <c r="H63" s="5" t="inlineStr">
@@ -3781,7 +3749,7 @@
       </c>
       <c r="K63" s="5" t="inlineStr">
         <is>
-          <t>Reference/QA only -- not unique across states, so never a merge key.</t>
+          <t>Reference only -- not unique across states, so never a merge key.</t>
         </is>
       </c>
     </row>
@@ -3814,7 +3782,7 @@
       </c>
       <c r="G64" s="5" t="inlineStr">
         <is>
-          <t>Derived from the daily extraction date</t>
+          <t>Daily extraction date</t>
         </is>
       </c>
       <c r="H64" s="5" t="inlineStr">
@@ -3824,7 +3792,7 @@
       </c>
       <c r="I64" s="5" t="inlineStr">
         <is>
-          <t>Parsed from the daily `date` column during aggregation</t>
+          <t>Parsed from the daily date column</t>
         </is>
       </c>
       <c r="J64" s="5" t="inlineStr">
@@ -3834,7 +3802,7 @@
       </c>
       <c r="K64" s="5" t="inlineStr">
         <is>
-          <t>45 years x 3,108 counties x 12 months = 1,678,320 rows in a complete build.</t>
+          <t>A complete build is 45 years x 3,108 counties x 12 months = 1,678,320 rows.</t>
         </is>
       </c>
     </row>
@@ -3867,7 +3835,7 @@
       </c>
       <c r="G65" s="5" t="inlineStr">
         <is>
-          <t>Derived from the daily extraction date</t>
+          <t>Daily extraction date</t>
         </is>
       </c>
       <c r="H65" s="5" t="inlineStr">
@@ -3877,7 +3845,7 @@
       </c>
       <c r="I65" s="5" t="inlineStr">
         <is>
-          <t>Parsed from the daily `date` column; becomes the j() variable in the SECTION 1/2 `reshape wide`</t>
+          <t>j() variable in the SECTION 1/2 reshape wide</t>
         </is>
       </c>
       <c r="J65" s="5" t="inlineStr">
@@ -3887,7 +3855,7 @@
       </c>
       <c r="K65" s="5" t="inlineStr">
         <is>
-          <t>Every monthly measure below appears in main_data_county_year.dta as 12 columns, &lt;var&gt;_m1 ... &lt;var&gt;_m12. The _m suffix was a 9/5/26 call (Stata's own reshape produces a bare `mean_temp_c1`).</t>
+          <t>Every monthly measure below appears in main_data_county_year.dta as 12 columns, &lt;var&gt;_m1 ... &lt;var&gt;_m12.</t>
         </is>
       </c>
     </row>
@@ -3920,7 +3888,7 @@
       </c>
       <c r="G66" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/ERA5/era5_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of ECMWF/ERA5_LAND/DAILY_AGGR via 04a_extract_era5_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/ERA5/extracted/county_daily_year)</t>
+          <t>dataRAW/ERA5/era5_county_daily_&lt;year&gt;.csv (GEE export of ECMWF/ERA5_LAND/DAILY_AGGR; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/ERA5/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H66" s="5" t="inlineStr">
@@ -3930,7 +3898,7 @@
       </c>
       <c r="I66" s="5" t="inlineStr">
         <is>
-          <t>count of daily rows in the geoid-year-month group (06)</t>
+          <t>Count of daily rows in the geoid-year-month group</t>
         </is>
       </c>
       <c r="J66" s="5" t="inlineStr">
@@ -3940,7 +3908,7 @@
       </c>
       <c r="K66" s="5" t="inlineStr">
         <is>
-          <t>Compare against expected_days; a short month means days were missing from the extract, not that the county had fewer days.</t>
+          <t>Compare against expected_days: a short month means days were missing from the extract.</t>
         </is>
       </c>
     </row>
@@ -3973,7 +3941,7 @@
       </c>
       <c r="G67" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/ERA5/era5_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of ECMWF/ERA5_LAND/DAILY_AGGR via 04a_extract_era5_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/ERA5/extracted/county_daily_year)</t>
+          <t>dataRAW/ERA5/era5_county_daily_&lt;year&gt;.csv (GEE export of ECMWF/ERA5_LAND/DAILY_AGGR; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/ERA5/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H67" s="5" t="inlineStr">
@@ -3983,7 +3951,7 @@
       </c>
       <c r="I67" s="5" t="inlineStr">
         <is>
-          <t>Identical logic to the PRISM block -- 06 runs one derivation against both datasets via DatasetConfig; only column names and units differ (precip_mm_total rather than ppt_total).</t>
+          <t>Identical logic to the PRISM block; only column names and units differ (precip_mm_total rather than ppt_total)</t>
         </is>
       </c>
       <c r="J67" s="5" t="inlineStr">
@@ -3993,7 +3961,7 @@
       </c>
       <c r="K67" s="5" t="inlineStr">
         <is>
-          <t>Exist for the PRISM-vs-ERA5 robustness comparison, not for the main panel. Do not merge them alongside the PRISM ones without renaming: the base names collide.</t>
+          <t>For the PRISM-vs-ERA5 robustness comparison, not the main panel. The base names collide with the PRISM columns.</t>
         </is>
       </c>
     </row>
@@ -4026,7 +3994,7 @@
       </c>
       <c r="G68" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/ERA5/era5_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of ECMWF/ERA5_LAND/DAILY_AGGR via 04a_extract_era5_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/ERA5/extracted/county_daily_year)</t>
+          <t>dataRAW/ERA5/era5_county_daily_&lt;year&gt;.csv (GEE export of ECMWF/ERA5_LAND/DAILY_AGGR; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/ERA5/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H68" s="5" t="inlineStr">
@@ -4036,17 +4004,17 @@
       </c>
       <c r="I68" s="5" t="inlineStr">
         <is>
-          <t>06: sum of daily snowfall_mm, grouped by geoid-year-month (thresholds live in SNOW_DEPTH_THRESHOLDS_IN). Stata SECTION 2 reshapes wide and renames to _m1.._m12.</t>
+          <t>06: sum of daily snowfall_mm, grouped by geoid-year-month (thresholds in SNOW_DEPTH_THRESHOLDS_IN); SECTION 2 reshapes wide and renames to _m1.._m12</t>
         </is>
       </c>
       <c r="J68" s="5" t="inlineStr">
         <is>
-          <t>Yes, reshaped wide as &lt;var&gt;_m1 .. &lt;var&gt;_m12 (SECTION 2)</t>
+          <t>Yes, as &lt;var&gt;_m1 .. &lt;var&gt;_m12 (SECTION 2)</t>
         </is>
       </c>
       <c r="K68" s="5" t="inlineStr">
         <is>
-          <t>PRISM has no snow variable at all, which is the whole reason ERA5 is merged into the weather panel. Missing readings compare False and contribute 0 to a count: geoid 25019 (Nantucket, MA) has no valid ERA5-Land land pixel at all, so its counts read 0 while mean_snow_depth is missing -- do not read a Nantucket WSI of 0 as a mild winter.</t>
+          <t>PRISM has no snow variable, which is why ERA5 is merged into the weather panel at all. Missing readings compare False and contribute 0 to a count -- see WEA-2 below.</t>
         </is>
       </c>
     </row>
@@ -4074,12 +4042,12 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>non-negative; metres (ERA5-Land native unit)</t>
+          <t>non-negative; metres (native ERA5-Land unit)</t>
         </is>
       </c>
       <c r="G69" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/ERA5/era5_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of ECMWF/ERA5_LAND/DAILY_AGGR via 04a_extract_era5_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/ERA5/extracted/county_daily_year)</t>
+          <t>dataRAW/ERA5/era5_county_daily_&lt;year&gt;.csv (GEE export of ECMWF/ERA5_LAND/DAILY_AGGR; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/ERA5/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H69" s="5" t="inlineStr">
@@ -4089,17 +4057,17 @@
       </c>
       <c r="I69" s="5" t="inlineStr">
         <is>
-          <t>06: mean of daily snow_depth, grouped by geoid-year-month (thresholds live in SNOW_DEPTH_THRESHOLDS_IN). Stata SECTION 2 reshapes wide and renames to _m1.._m12.</t>
+          <t>06: mean of daily snow_depth, grouped by geoid-year-month (thresholds in SNOW_DEPTH_THRESHOLDS_IN); SECTION 2 reshapes wide and renames to _m1.._m12</t>
         </is>
       </c>
       <c r="J69" s="5" t="inlineStr">
         <is>
-          <t>Yes, reshaped wide as &lt;var&gt;_m1 .. &lt;var&gt;_m12 (SECTION 2)</t>
+          <t>Yes, as &lt;var&gt;_m1 .. &lt;var&gt;_m12 (SECTION 2)</t>
         </is>
       </c>
       <c r="K69" s="5" t="inlineStr">
         <is>
-          <t>A stock, so averaged not summed. Cannot substitute for the day counts below: a month can average under a threshold and still contain qualifying days. Missing readings compare False and contribute 0 to a count: geoid 25019 (Nantucket, MA) has no valid ERA5-Land land pixel at all, so its counts read 0 while mean_snow_depth is missing -- do not read a Nantucket WSI of 0 as a mild winter.</t>
+          <t>A stock, so averaged not summed. Cannot substitute for the day counts below: a month can average under a threshold and still contain qualifying days. Missing readings compare False and contribute 0 to a count -- see WEA-2 below.</t>
         </is>
       </c>
     </row>
@@ -4132,7 +4100,7 @@
       </c>
       <c r="G70" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/ERA5/era5_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of ECMWF/ERA5_LAND/DAILY_AGGR via 04a_extract_era5_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/ERA5/extracted/county_daily_year)</t>
+          <t>dataRAW/ERA5/era5_county_daily_&lt;year&gt;.csv (GEE export of ECMWF/ERA5_LAND/DAILY_AGGR; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/ERA5/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H70" s="5" t="inlineStr">
@@ -4142,17 +4110,17 @@
       </c>
       <c r="I70" s="5" t="inlineStr">
         <is>
-          <t>06: count of daily snow_depth &gt;= 18*0.0254m, grouped by geoid-year-month (thresholds live in SNOW_DEPTH_THRESHOLDS_IN). Stata SECTION 2 reshapes wide and renames to _m1.._m12.</t>
+          <t>06: count of daily snow_depth &gt;= 18*0.0254m, grouped by geoid-year-month (thresholds in SNOW_DEPTH_THRESHOLDS_IN); SECTION 2 reshapes wide and renames to _m1.._m12</t>
         </is>
       </c>
       <c r="J70" s="5" t="inlineStr">
         <is>
-          <t>Yes, reshaped wide as &lt;var&gt;_m1 .. &lt;var&gt;_m12 (SECTION 2)</t>
+          <t>Yes, as &lt;var&gt;_m1 .. &lt;var&gt;_m12 (SECTION 2)</t>
         </is>
       </c>
       <c r="K70" s="5" t="inlineStr">
         <is>
-          <t>Kohn (1975) / WI DNR literature threshold and the snow-hazard component of the WSI (wsi_snow_days). INCLUSIVE (&gt;=), matching '18 or more inches of snow on the ground'. County-averaged ERA5-Land snow depth strips out the local maxima an 18in cutoff was calibrated on: on the 1981 extract Wisconsin recorded 8 county-days &gt;=18in statewide (all Vilas County) and MN/IA/IL/PA none, so the index is driven almost entirely by its cold component across most of the study area. Missing readings compare False and contribute 0 to a count: geoid 25019 (Nantucket, MA) has no valid ERA5-Land land pixel at all, so its counts read 0 while mean_snow_depth is missing -- do not read a Nantucket WSI of 0 as a mild winter.</t>
+          <t>Kohn (1975) / WI DNR threshold and the WSI's snow component (wsi_snow_days). INCLUSIVE (&gt;=). County-averaged ERA5-Land snow depth strips out the local maxima an 18in cutoff was calibrated on, so this is near-zero across most of the eastern deer range -- see WEA-1 below. Missing readings compare False and contribute 0 to a count -- see WEA-2 below.</t>
         </is>
       </c>
     </row>
@@ -4185,7 +4153,7 @@
       </c>
       <c r="G71" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/ERA5/era5_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of ECMWF/ERA5_LAND/DAILY_AGGR via 04a_extract_era5_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/ERA5/extracted/county_daily_year)</t>
+          <t>dataRAW/ERA5/era5_county_daily_&lt;year&gt;.csv (GEE export of ECMWF/ERA5_LAND/DAILY_AGGR; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/ERA5/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H71" s="5" t="inlineStr">
@@ -4195,17 +4163,17 @@
       </c>
       <c r="I71" s="5" t="inlineStr">
         <is>
-          <t>06: count of daily snow_depth &gt;= 12*0.0254m, grouped by geoid-year-month (thresholds live in SNOW_DEPTH_THRESHOLDS_IN). Stata SECTION 2 reshapes wide and renames to _m1.._m12.</t>
+          <t>06: count of daily snow_depth &gt;= 12*0.0254m, grouped by geoid-year-month (thresholds in SNOW_DEPTH_THRESHOLDS_IN); SECTION 2 reshapes wide and renames to _m1.._m12</t>
         </is>
       </c>
       <c r="J71" s="5" t="inlineStr">
         <is>
-          <t>Yes, reshaped wide as &lt;var&gt;_m1 .. &lt;var&gt;_m12 (SECTION 2)</t>
+          <t>Yes, as &lt;var&gt;_m1 .. &lt;var&gt;_m12 (SECTION 2)</t>
         </is>
       </c>
       <c r="K71" s="5" t="inlineStr">
         <is>
-          <t>A sensitivity variant, NOT a competing definition of the Kohn index. Report winter_severity_index; use this for the robustness table. Missing readings compare False and contribute 0 to a count: geoid 25019 (Nantucket, MA) has no valid ERA5-Land land pixel at all, so its counts read 0 while mean_snow_depth is missing -- do not read a Nantucket WSI of 0 as a mild winter.</t>
+          <t>A sensitivity variant, not a competing definition of the Kohn index. Missing readings compare False and contribute 0 to a count -- see WEA-2 below.</t>
         </is>
       </c>
     </row>
@@ -4238,7 +4206,7 @@
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>dataRAW/ERA5/era5_county_daily_&lt;year&gt;_&lt;stamp&gt;.csv (GEE export of ECMWF/ERA5_LAND/DAILY_AGGR via 04a_extract_era5_county.py; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/ERA5/extracted/county_daily_year)</t>
+          <t>dataRAW/ERA5/era5_county_daily_&lt;year&gt;.csv (GEE export of ECMWF/ERA5_LAND/DAILY_AGGR; on Kodama /mnt/data_f/AnimalCollisionsWeatherData/ERA5/extracted/county_daily_year)</t>
         </is>
       </c>
       <c r="H72" s="5" t="inlineStr">
@@ -4248,17 +4216,17 @@
       </c>
       <c r="I72" s="5" t="inlineStr">
         <is>
-          <t>06: count of daily snow_depth &gt;= 8*0.0254m, grouped by geoid-year-month (thresholds live in SNOW_DEPTH_THRESHOLDS_IN). Stata SECTION 2 reshapes wide and renames to _m1.._m12.</t>
+          <t>06: count of daily snow_depth &gt;= 8*0.0254m, grouped by geoid-year-month (thresholds in SNOW_DEPTH_THRESHOLDS_IN); SECTION 2 reshapes wide and renames to _m1.._m12</t>
         </is>
       </c>
       <c r="J72" s="5" t="inlineStr">
         <is>
-          <t>Yes, reshaped wide as &lt;var&gt;_m1 .. &lt;var&gt;_m12 (SECTION 2)</t>
+          <t>Yes, as &lt;var&gt;_m1 .. &lt;var&gt;_m12 (SECTION 2)</t>
         </is>
       </c>
       <c r="K72" s="5" t="inlineStr">
         <is>
-          <t>Same status as the 12in variant. Missing readings compare False and contribute 0 to a count: geoid 25019 (Nantucket, MA) has no valid ERA5-Land land pixel at all, so its counts read 0 while mean_snow_depth is missing -- do not read a Nantucket WSI of 0 as a mild winter.</t>
+          <t>Same status as the 12in variant. Missing readings compare False and contribute 0 to a count -- see WEA-2 below.</t>
         </is>
       </c>
     </row>
@@ -4301,7 +4269,7 @@
       </c>
       <c r="I73" s="5" t="inlineStr">
         <is>
-          <t>Not kept by SECTION 2's `keep`</t>
+          <t>Not kept by SECTION 2</t>
         </is>
       </c>
       <c r="J73" s="5" t="inlineStr">
@@ -4309,11 +4277,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="K73" s="5" t="inlineStr">
-        <is>
-          <t>ERA5's only incomplete-month source is the Nantucket gap (16,436 missing daily readings, all geoid 25019).</t>
-        </is>
-      </c>
+      <c r="K73" s="5" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
@@ -4349,7 +4313,7 @@
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>dataCSV/PRISM/prism_derived_weather_vars.csv and dataCSV/ERA5/era5_derived_weather_vars.csv (codePYTHON/06), which in turn come from the daily GEE extracts</t>
+          <t>dataCSV/PRISM/prism_derived_weather_vars.csv and dataCSV/ERA5/era5_derived_weather_vars.csv (06)</t>
         </is>
       </c>
       <c r="H74" s="5" t="inlineStr">
@@ -4359,7 +4323,7 @@
       </c>
       <c r="I74" s="5" t="inlineStr">
         <is>
-          <t>Carried through from the derived-vars files; imported with stringcols(1) in SECTION 7</t>
+          <t>Imported with stringcols(1) in SECTION 7</t>
         </is>
       </c>
       <c r="J74" s="5" t="inlineStr">
@@ -4369,7 +4333,7 @@
       </c>
       <c r="K74" s="5" t="inlineStr">
         <is>
-          <t>This file has only geoid and year -- no state_fips/county_fips/county_name, since it is merged onto a panel that already has them.</t>
+          <t>This file carries only geoid and year -- it is merged onto a panel that already has the other identifiers.</t>
         </is>
       </c>
     </row>
@@ -4402,7 +4366,7 @@
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>dataCSV/PRISM/prism_derived_weather_vars.csv and dataCSV/ERA5/era5_derived_weather_vars.csv (codePYTHON/06), which in turn come from the daily GEE extracts</t>
+          <t>dataCSV/PRISM/prism_derived_weather_vars.csv and dataCSV/ERA5/era5_derived_weather_vars.csv (06)</t>
         </is>
       </c>
       <c r="H75" s="5" t="inlineStr">
@@ -4422,7 +4386,7 @@
       </c>
       <c r="K75" s="5" t="inlineStr">
         <is>
-          <t>WIDER than the 3-month DJF window mean_winter_temp uses. Year t is missing wherever December of t-1 is out of panel, including the panel's first year -- the same behaviour the old L1. construction produced.</t>
+          <t>WIDER than the 3-month DJF window mean_winter_temp uses. Year t is missing wherever December of t-1 is out of panel, including the panel's first year.</t>
         </is>
       </c>
     </row>
@@ -4440,12 +4404,12 @@
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>days</t>
+          <t>numeric (int)</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t>numeric (int)</t>
+          <t>county-winter-year (winter t = Dec of t-1 through Apr of t)</t>
         </is>
       </c>
       <c r="F76" s="5" t="inlineStr">
@@ -4455,7 +4419,7 @@
       </c>
       <c r="G76" s="5" t="inlineStr">
         <is>
-          <t>dataCSV/PRISM/prism_derived_weather_vars.csv and dataCSV/ERA5/era5_derived_weather_vars.csv (codePYTHON/06), which in turn come from the daily GEE extracts</t>
+          <t>dataCSV/PRISM/prism_derived_weather_vars.csv and dataCSV/ERA5/era5_derived_weather_vars.csv (06)</t>
         </is>
       </c>
       <c r="H76" s="5" t="inlineStr">
@@ -4465,7 +4429,7 @@
       </c>
       <c r="I76" s="5" t="inlineStr">
         <is>
-          <t>06c: seasonal sum of days_extremely_cold over months 12 (prior year), 1, 2, 3, 4. Missing propagates -- any of the five months absent makes the season NaN, not a partial sum (matching Stata's gen).</t>
+          <t>06c: seasonal sum of days_extremely_cold over months 12 (prior year), 1, 2, 3, 4. Missing propagates -- any of the five months absent makes the season missing, not a partial sum.</t>
         </is>
       </c>
       <c r="J76" s="5" t="inlineStr">
@@ -4473,11 +4437,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K76" s="5" t="inlineStr">
-        <is>
-          <t>Built in Python since 09/17/2026; before that it was SECTION 7 of the merge script, which made a Phase 4 exhibit (09b) depend on a Phase 6 output. Definition ported unchanged and verified county-by-county against the old output.</t>
-        </is>
-      </c>
+      <c r="K76" s="5" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="5" t="n"/>
@@ -4493,12 +4453,12 @@
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>days</t>
+          <t>numeric (int)</t>
         </is>
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t>numeric (int)</t>
+          <t>county-winter-year (winter t = Dec of t-1 through Apr of t)</t>
         </is>
       </c>
       <c r="F77" s="5" t="inlineStr">
@@ -4508,7 +4468,7 @@
       </c>
       <c r="G77" s="5" t="inlineStr">
         <is>
-          <t>dataCSV/PRISM/prism_derived_weather_vars.csv and dataCSV/ERA5/era5_derived_weather_vars.csv (codePYTHON/06), which in turn come from the daily GEE extracts</t>
+          <t>dataCSV/PRISM/prism_derived_weather_vars.csv and dataCSV/ERA5/era5_derived_weather_vars.csv (06)</t>
         </is>
       </c>
       <c r="H77" s="5" t="inlineStr">
@@ -4528,7 +4488,7 @@
       </c>
       <c r="K77" s="5" t="inlineStr">
         <is>
-          <t>Near-degenerate across most of the eastern deer range because of county-level spatial averaging -- see open item WEA-3 below.</t>
+          <t>Near-zero across most of the eastern deer range -- see WEA-1 below.</t>
         </is>
       </c>
     </row>
@@ -4546,12 +4506,12 @@
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>days</t>
+          <t>numeric (int)</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t>numeric (int)</t>
+          <t>county-winter-year (winter t = Dec of t-1 through Apr of t)</t>
         </is>
       </c>
       <c r="F78" s="5" t="inlineStr">
@@ -4561,7 +4521,7 @@
       </c>
       <c r="G78" s="5" t="inlineStr">
         <is>
-          <t>dataCSV/PRISM/prism_derived_weather_vars.csv and dataCSV/ERA5/era5_derived_weather_vars.csv (codePYTHON/06), which in turn come from the daily GEE extracts</t>
+          <t>dataCSV/PRISM/prism_derived_weather_vars.csv and dataCSV/ERA5/era5_derived_weather_vars.csv (06)</t>
         </is>
       </c>
       <c r="H78" s="5" t="inlineStr">
@@ -4581,7 +4541,7 @@
       </c>
       <c r="K78" s="5" t="inlineStr">
         <is>
-          <t>Robustness only. NOT alternative definitions of the Kohn index.</t>
+          <t>Robustness only, not alternative definitions of the index.</t>
         </is>
       </c>
     </row>
@@ -4599,22 +4559,22 @@
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>points</t>
+          <t>numeric (int)</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t>numeric (int)</t>
+          <t>county-winter-year (winter t = Dec of t-1 through Apr of t)</t>
         </is>
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>0-302; categories &lt;50 mild, 50-80 moderate, 80-100 moderately severe, &gt;100 very severe</t>
+          <t>0-302; &lt;50 mild, 50-80 moderate, 80-100 moderately severe, &gt;100 very severe</t>
         </is>
       </c>
       <c r="G79" s="5" t="inlineStr">
         <is>
-          <t>dataCSV/PRISM/prism_derived_weather_vars.csv and dataCSV/ERA5/era5_derived_weather_vars.csv (codePYTHON/06), which in turn come from the daily GEE extracts</t>
+          <t>dataCSV/PRISM/prism_derived_weather_vars.csv and dataCSV/ERA5/era5_derived_weather_vars.csv (06)</t>
         </is>
       </c>
       <c r="H79" s="5" t="inlineStr">
@@ -4634,7 +4594,7 @@
       </c>
       <c r="K79" s="5" t="inlineStr">
         <is>
-          <t>A day meeting both conditions counts in both tallies -- that is the literature's 'adds 2 points' rule, not double counting. This is the variable to report.</t>
+          <t>A day meeting both conditions counts in both tallies -- the literature's 'adds 2 points' rule, not double counting. This is the variable to report.</t>
         </is>
       </c>
     </row>
@@ -4652,12 +4612,12 @@
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>points</t>
+          <t>numeric (int)</t>
         </is>
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t>numeric (int)</t>
+          <t>county-winter-year (winter t = Dec of t-1 through Apr of t)</t>
         </is>
       </c>
       <c r="F80" s="5" t="inlineStr">
@@ -4667,7 +4627,7 @@
       </c>
       <c r="G80" s="5" t="inlineStr">
         <is>
-          <t>dataCSV/PRISM/prism_derived_weather_vars.csv and dataCSV/ERA5/era5_derived_weather_vars.csv (codePYTHON/06), which in turn come from the daily GEE extracts</t>
+          <t>dataCSV/PRISM/prism_derived_weather_vars.csv and dataCSV/ERA5/era5_derived_weather_vars.csv (06)</t>
         </is>
       </c>
       <c r="H80" s="5" t="inlineStr">
@@ -4705,7 +4665,7 @@
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>5-digit county FIPS (2-digit state + 3-digit county); the canonical merge key against every other RA's county-level panel</t>
+          <t>5-digit county FIPS (state + county); the merge key against every other county-level panel</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
@@ -4725,7 +4685,7 @@
       </c>
       <c r="G81" s="5" t="inlineStr">
         <is>
-          <t>Census: PE-02 flat files (1981-89); intercensal API int_charagegroups (1990-99); CO-EST00INT (2000-09); CC-EST2020INT (2010-20); CC-EST2025 (2020-25). Cached under dataRAW/Population/&lt;source&gt;/</t>
+          <t>Census: PE-02 flat files (1981-89); intercensal API int_charagegroups (1990-99); CO-EST00INT (2000-09); CC-EST2020INT (2010-20); CC-EST2025 (2020-25). Cached under dataRAW/Population/</t>
         </is>
       </c>
       <c r="H81" s="5" t="inlineStr">
@@ -4735,7 +4695,7 @@
       </c>
       <c r="I81" s="5" t="inlineStr">
         <is>
-          <t>Written by the GEE extraction; imported into Stata with stringcols(1 2 3) so leading zeros survive</t>
+          <t>Imported with stringcols(1 2 3) so leading zeros survive</t>
         </is>
       </c>
       <c r="J81" s="5" t="inlineStr">
@@ -4745,7 +4705,7 @@
       </c>
       <c r="K81" s="5" t="inlineStr">
         <is>
-          <t>Text, not numeric -- leading zeros are meaningful. Merge on geoid, never on county_name (names are not unique across states). County universe is TIGER/2018 everywhere in this pipeline. Population is recoded FORWARD onto TIGER/2018 so it keys to the same county universe as the weather panel.</t>
+          <t>Text, not numeric. Merge on geoid, never on county_name. County universe is TIGER/2018 throughout. Population is recoded forward onto TIGER/2018, so it keys to the same county universe as the weather panel.</t>
         </is>
       </c>
     </row>
@@ -4778,7 +4738,7 @@
       </c>
       <c r="G82" s="5" t="inlineStr">
         <is>
-          <t>TIGER/2018/Counties (Earth Engine FeatureCollection), carried through the GEE extraction</t>
+          <t>TIGER/2018/Counties (Earth Engine FeatureCollection)</t>
         </is>
       </c>
       <c r="H82" s="5" t="inlineStr">
@@ -4788,7 +4748,7 @@
       </c>
       <c r="I82" s="5" t="inlineStr">
         <is>
-          <t>Carried through from the extraction; stringcols on import</t>
+          <t>Carried through from the extraction</t>
         </is>
       </c>
       <c r="J82" s="5" t="inlineStr">
@@ -4796,11 +4756,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K82" s="5" t="inlineStr">
-        <is>
-          <t>CONUS scope is defined once, in gee_extract_utils.CONUS_STATE_FIPS, and imported by every extraction script.</t>
-        </is>
-      </c>
+      <c r="K82" s="5" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="5" t="n"/>
@@ -4831,7 +4787,7 @@
       </c>
       <c r="G83" s="5" t="inlineStr">
         <is>
-          <t>TIGER/2018/Counties (Earth Engine FeatureCollection), carried through the GEE extraction</t>
+          <t>TIGER/2018/Counties (Earth Engine FeatureCollection)</t>
         </is>
       </c>
       <c r="H83" s="5" t="inlineStr">
@@ -4841,7 +4797,7 @@
       </c>
       <c r="I83" s="5" t="inlineStr">
         <is>
-          <t>Carried through from the extraction; stringcols on import</t>
+          <t>Carried through from the extraction</t>
         </is>
       </c>
       <c r="J83" s="5" t="inlineStr">
@@ -4849,11 +4805,7 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K83" s="5" t="inlineStr">
-        <is>
-          <t>Combine with state_fips for a nationally unique key, or just use geoid.</t>
-        </is>
-      </c>
+      <c r="K83" s="5" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="5" t="n"/>
@@ -4884,7 +4836,7 @@
       </c>
       <c r="G84" s="5" t="inlineStr">
         <is>
-          <t>TIGER/2018/Counties (Earth Engine FeatureCollection), carried through the GEE extraction</t>
+          <t>TIGER/2018/Counties (Earth Engine FeatureCollection)</t>
         </is>
       </c>
       <c r="H84" s="5" t="inlineStr">
@@ -4904,7 +4856,7 @@
       </c>
       <c r="K84" s="5" t="inlineStr">
         <is>
-          <t>Reference/QA only -- not unique across states, so never a merge key.</t>
+          <t>Reference only -- not unique across states, so never a merge key.</t>
         </is>
       </c>
     </row>
@@ -4937,7 +4889,7 @@
       </c>
       <c r="G85" s="5" t="inlineStr">
         <is>
-          <t>Census: PE-02 flat files (1981-89); intercensal API int_charagegroups (1990-99); CO-EST00INT (2000-09); CC-EST2020INT (2010-20); CC-EST2025 (2020-25). Cached under dataRAW/Population/&lt;source&gt;/</t>
+          <t>Census: PE-02 flat files (1981-89); intercensal API int_charagegroups (1990-99); CO-EST00INT (2000-09); CC-EST2020INT (2010-20); CC-EST2025 (2020-25). Cached under dataRAW/Population/</t>
         </is>
       </c>
       <c r="H85" s="5" t="inlineStr">
@@ -4947,7 +4899,7 @@
       </c>
       <c r="I85" s="5" t="inlineStr">
         <is>
-          <t>08b: normalized from each product's own YEAR code, which means three different things across the five sources (YEAR_CODE_RULES; co-est00int needs an explicit map because it carries a 4/1/2010 census row in the MIDDLE of its code sequence).</t>
+          <t>08b normalizes each product's own YEAR code, which means three different things across the five sources (co-est00int needs an explicit map -- it carries a 4/1/2010 census row in the middle of its code sequence)</t>
         </is>
       </c>
       <c r="J85" s="5" t="inlineStr">
@@ -4957,7 +4909,7 @@
       </c>
       <c r="K85" s="5" t="inlineStr">
         <is>
-          <t>Estimates are July 1 of the stated year, EXCEPT 2020, which comes from the 2010-2020 intercensal and is the 4/1/2020 census count. ~0.2% effect; still undocumented in the appendix and never put to the PI.</t>
+          <t>Estimates are July 1 of the stated year, except 2020, which is the 4/1/2020 census count (~0.2% difference).</t>
         </is>
       </c>
     </row>
@@ -5000,7 +4952,7 @@
       </c>
       <c r="I86" s="5" t="inlineStr">
         <is>
-          <t>08b five stages in order: fetch (never recodes geography) -&gt; stack (never dedupes silently) -&gt; crosswalk (the only stage that changes a geoid) -&gt; CT override -&gt; validate (never mutates). Merged into the main panel 1:1 on geoid year in SECTION 3, with no assert/drop on _merge (settled 9/1/26).</t>
+          <t>08b: fetch -&gt; stack -&gt; FIPS crosswalk -&gt; CT override -&gt; validate. SECTION 3 merges it 1:1 on geoid year, keeping unmatched rows on both sides rather than asserting _merge==3.</t>
         </is>
       </c>
       <c r="J86" s="5" t="inlineStr">
@@ -5010,7 +4962,7 @@
       </c>
       <c r="K86" s="5" t="inlineStr">
         <is>
-          <t>One vintage per period, never spliced mid-decade. Everything except 2020-25 is intercensal (final, reconciled to the decennial count at both ends of its decade); 2020-25 is POSTCENSAL and provisional until the 2030 census anchors it. National totals track the decennial counts at 1990/2000/2010/2020 to within the AK+HI exclusion plus the July-vs-April offset.</t>
+          <t>One vintage per period, never spliced mid-decade. 1981-2019 is intercensal (final, reconciled to the decennial count at both ends of its decade); 2020-2025 is postcensal and provisional until the 2030 census anchors it. National totals track the decennial counts at 1990/2000/2010/2020 to within the AK+HI exclusion and the July-vs-April offset.</t>
         </is>
       </c>
     </row>
@@ -5053,7 +5005,7 @@
       </c>
       <c r="I87" s="5" t="inlineStr">
         <is>
-          <t>08b: compute_age_shares() pivots the normalized AGEGRP detail and divides by the county-year total. AGEGRP encoding is DETECTED from the data (does code 0 equal the sum of 1-18?), normalized, then re-asserted for every source with no exceptions.</t>
+          <t>08b: compute_age_shares() pivots the normalized AGEGRP detail and divides by the county-year total. The AGEGRP convention is detected from the data, normalized, then re-asserted for every source.</t>
         </is>
       </c>
       <c r="J87" s="5" t="inlineStr">
@@ -5063,7 +5015,7 @@
       </c>
       <c r="K87" s="5" t="inlineStr">
         <is>
-          <t>Time-varying regression controls, added per the 9/1/26 guidance. Sex and race are collapsed, never broken out. AGEGRP means three different things across the five products; a mis-read of co-est00int's code 99 total once made the whole 2000s decade 70x wrong while every structural check passed -- see project memory census-encoding-traps.</t>
+          <t>Time-varying regression controls. Sex and race are collapsed, never broken out. AGEGRP means three different things across the five products and a misread of one of them is invisible to structural checks -- do not add a source without running the encoding guard.</t>
         </is>
       </c>
     </row>
@@ -5091,12 +5043,12 @@
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>census_intercensal_api_1990s / census_intercensal_2000s / census_intercensal_2010s / census_postcensal_2020s / ct_town_reaggregation / (blank where population is missing)</t>
+          <t>census_intercensal_api_1990s / census_intercensal_2000s / census_intercensal_2010s / census_postcensal_2020s / ct_town_reaggregation / blank where population is missing</t>
         </is>
       </c>
       <c r="G88" s="5" t="inlineStr">
         <is>
-          <t>Census: PE-02 flat files (1981-89); intercensal API int_charagegroups (1990-99); CO-EST00INT (2000-09); CC-EST2020INT (2010-20); CC-EST2025 (2020-25). Cached under dataRAW/Population/&lt;source&gt;/</t>
+          <t>Census: PE-02 flat files (1981-89); intercensal API int_charagegroups (1990-99); CO-EST00INT (2000-09); CC-EST2020INT (2010-20); CC-EST2025 (2020-25). Cached under dataRAW/Population/</t>
         </is>
       </c>
       <c r="H88" s="5" t="inlineStr">
@@ -5116,7 +5068,7 @@
       </c>
       <c r="K88" s="5" t="inlineStr">
         <is>
-          <t>Lets any result be traced back to a vintage. ct_town_reaggregation marks the 40 CT county-years supplied by 08a.</t>
+          <t>Lets any figure be traced to a vintage. ct_town_reaggregation marks the CT county-years supplied by 08a.</t>
         </is>
       </c>
     </row>
@@ -5149,7 +5101,7 @@
       </c>
       <c r="G89" s="5" t="inlineStr">
         <is>
-          <t>Census: PE-02 flat files (1981-89); intercensal API int_charagegroups (1990-99); CO-EST00INT (2000-09); CC-EST2020INT (2010-20); CC-EST2025 (2020-25). Cached under dataRAW/Population/&lt;source&gt;/</t>
+          <t>Census: PE-02 flat files (1981-89); intercensal API int_charagegroups (1990-99); CO-EST00INT (2000-09); CC-EST2020INT (2010-20); CC-EST2025 (2020-25). Cached under dataRAW/Population/</t>
         </is>
       </c>
       <c r="H89" s="5" t="inlineStr">
@@ -5197,7 +5149,7 @@
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>blank (111,820 of 111,888 rows in the 1990-2025 build); 'includes territory that became 08014 in 2001; discontinuity at 2001' (44); 'excludes 30113, which was absorbed in 1997 and is not separable' (14); 'county created 2001 from parts of other counties; no separable population exists at county level before then' (10)</t>
+          <t>blank; 'includes territory that became 08014 in 2001; discontinuity at 2001'; 'excludes 30113, which was absorbed in 1997 and is not separable'; 'county created 2001 from parts of other counties; no separable population exists at county level before then'</t>
         </is>
       </c>
       <c r="G90" s="5" t="inlineStr">
@@ -5212,7 +5164,7 @@
       </c>
       <c r="I90" s="5" t="inlineStr">
         <is>
-          <t>Set by apply_fips_crosswalk where a FIPS change cannot be cleanly apportioned</t>
+          <t>Set where a FIPS change cannot be cleanly apportioned</t>
         </is>
       </c>
       <c r="J90" s="5" t="inlineStr">
@@ -5222,7 +5174,7 @@
       </c>
       <c r="K90" s="5" t="inlineStr">
         <is>
-          <t>The three flag texts are exactly the three unapportionable changes in the window: Broomfield CO 08014 (created 2001 from four parents; left NaN rather than back-apportioned, because the area had no separate collisions either and a back-cast denominator would produce a fake near-zero rate for two decades), its four parents, and the Yellowstone 30113 merge_split. Review rows are also written to population_review_flags.csv.</t>
+          <t>The three texts cover the three unapportionable changes in the window: Broomfield CO 08014, its four parent counties, and the Yellowstone 30113 split. Flagged rows are also written to population_review_flags.csv. Treat flagged county-years with care in any per-capita denominator.</t>
         </is>
       </c>
     </row>
@@ -5250,7 +5202,7 @@
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
-          <t>blank; 'age detail unavailable or does not sum to 1' (40 rows = CT 2021-2025)</t>
+          <t>blank; 'age detail unavailable or does not sum to 1' (CT 2021-2025, 40 rows)</t>
         </is>
       </c>
       <c r="G91" s="5" t="inlineStr">
@@ -5275,7 +5227,7 @@
       </c>
       <c r="K91" s="5" t="inlineStr">
         <is>
-          <t>The 40 flagged rows are CT 2021-25, where 08a supplies totals only. Census publishes sub-county population as totals in every vintage and CT DPH town-level age data is not annual, so these are genuinely unavailable -- do NOT model them down.</t>
+          <t>The flagged rows are genuinely unavailable, not a build gap -- do not model them down.</t>
         </is>
       </c>
     </row>
@@ -5293,7 +5245,7 @@
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>CT legacy-county identifiers (the 8 counties, 09001-09015)</t>
+          <t>CT legacy-county identifiers (the 8 counties)</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr">
@@ -5313,7 +5265,7 @@
       </c>
       <c r="G92" s="5" t="inlineStr">
         <is>
-          <t>2018 Gazetteer county-subdivision file (town -&gt; county mapping, joined on COUSUB FIPS, not on town name)</t>
+          <t>2018 Gazetteer county-subdivision file (town -&gt; county mapping, joined on COUSUB FIPS, not town name)</t>
         </is>
       </c>
       <c r="H92" s="5" t="inlineStr">
@@ -5323,17 +5275,17 @@
       </c>
       <c r="I92" s="5" t="inlineStr">
         <is>
-          <t>08a: town-level population aggregated up through a static pre-2022 town-&gt;county mapping</t>
+          <t>08a aggregates town-level population up through a static pre-2022 town-&gt;county mapping</t>
         </is>
       </c>
       <c r="J92" s="5" t="inlineStr">
         <is>
-          <t>Yes -- via 08b, which overrides its own CT rows with this file</t>
+          <t>Yes, via 08b, which overrides its own CT rows with this file</t>
         </is>
       </c>
       <c r="K92" s="5" t="inlineStr">
         <is>
-          <t>Census's Vintage 2022+ estimates report CT as 9 planning regions (09110-09190), which do NOT nest inside the 8 legacy counties. Both schemes are just different aggregations of the same 169 towns, so going through towns sidesteps the non-nesting problem. THIS DESIGN IS NOT RATIFIED BY THE PI.</t>
+          <t>Census's Vintage 2022+ estimates report CT as 9 planning regions, which do not nest inside the 8 legacy counties. Both schemes are aggregations of the same 169 towns, so going through towns sidesteps the non-nesting problem.</t>
         </is>
       </c>
     </row>
@@ -5376,17 +5328,17 @@
       </c>
       <c r="I93" s="5" t="inlineStr">
         <is>
-          <t>Production scope; 2015 and 2018 are run as VALIDATION years only (cross_check_against_direct_county_pull), where Census still published legacy counties so the two methods can be compared</t>
+          <t>Production scope; 2015 and 2018 are run as validation years only, where Census still published legacy counties and the two methods can be compared</t>
         </is>
       </c>
       <c r="J93" s="5" t="inlineStr">
         <is>
-          <t>No (validation years are not written to production)</t>
+          <t>No (validation years are not written)</t>
         </is>
       </c>
       <c r="K93" s="5" t="inlineStr">
         <is>
-          <t>Scope was 2022-2025 until 09/04/2026: cc-est2025 reports planning regions for EVERY year it covers, 2020-2025, so 2021 fell through as 8 missing county-years in the first full build. 2020 is rescued by the intercensal file.</t>
+          <t>2020 comes from the intercensal file, not from here.</t>
         </is>
       </c>
     </row>
@@ -5429,17 +5381,17 @@
       </c>
       <c r="I94" s="5" t="inlineStr">
         <is>
-          <t>Sum of the 169 towns' population within each legacy county</t>
+          <t>Sum of the 169 towns within each legacy county</t>
         </is>
       </c>
       <c r="J94" s="5" t="inlineStr">
         <is>
-          <t>Yes (as population, with population_source = ct_town_reaggregation)</t>
+          <t>Yes (population_source = ct_town_reaggregation)</t>
         </is>
       </c>
       <c r="K94" s="5" t="inlineStr">
         <is>
-          <t>TOTALS ONLY -- no age detail, hence the 40 age_flag rows above. Cross-check against a direct county pull agreed within 0.1% at 2015 and 2018.</t>
+          <t>Totals only, no age detail -- the source of the 40 age_flag rows. Cross-check against a direct county pull agreed within 0.1% at 2015 and 2018.</t>
         </is>
       </c>
     </row>
@@ -5496,7 +5448,7 @@
       <c r="A96" s="4" t="inlineStr">
         <is>
           <t>fips_crosswalk_1980_2025.csv
-(hand-maintained input to 08b)</t>
+(input to 08b)</t>
         </is>
       </c>
       <c r="B96" s="4" t="inlineStr">
@@ -5521,12 +5473,12 @@
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
-          <t>10 rows total; blank for splits, by design</t>
+          <t>10 rows; blank on split rows by design</t>
         </is>
       </c>
       <c r="G96" s="5" t="inlineStr">
         <is>
-          <t>Census 'Substantial Changes to Counties and County Equivalent Entities' decade pages (1980-2020), read directly; cross-checked against David Dorn's FIPS County Code Changes (May 2007, rev. Sept 2021)</t>
+          <t>Census 'Substantial Changes to Counties and County Equivalent Entities' decade pages (1980-2020), cross-checked against Dorn's FIPS County Code Changes</t>
         </is>
       </c>
       <c r="H96" s="5" t="inlineStr">
@@ -5536,7 +5488,7 @@
       </c>
       <c r="I96" s="5" t="inlineStr">
         <is>
-          <t>Hand-compiled and verified 9/3/26; consumed by population_utils.apply_fips_crosswalk</t>
+          <t>Consumed by population_utils.apply_fips_crosswalk</t>
         </is>
       </c>
       <c r="J96" s="5" t="inlineStr">
@@ -5546,7 +5498,7 @@
       </c>
       <c r="K96" s="5" t="inlineStr">
         <is>
-          <t>Blank on split rows because there is no single valid source county; parent FIPS are written in `notes` in parentheses, which is where _parse_parent_geoids reads them from.</t>
+          <t>Blank on splits because there is no single valid source county; parent FIPS are written in notes in parentheses, where _parse_parent_geoids reads them from.</t>
         </is>
       </c>
     </row>
@@ -5589,7 +5541,7 @@
       </c>
       <c r="I97" s="5" t="inlineStr">
         <is>
-          <t>Everything is recoded FORWARD onto TIGER/2018</t>
+          <t>Everything is recoded forward onto TIGER/2018</t>
         </is>
       </c>
       <c r="J97" s="5" t="inlineStr">
@@ -5599,7 +5551,7 @@
       </c>
       <c r="K97" s="5" t="inlineStr">
         <is>
-          <t>Dorn harmonizes the OTHER way (modern codes back onto 1980-era codes, because his target is 1990 commuting zones). We take his change list, not his direction -- do not 'fix' this back after reading him.</t>
+          <t>Dorn harmonizes the other way (modern codes back onto 1980-era codes, for 1990 commuting zones). We take his change list, not his direction.</t>
         </is>
       </c>
     </row>
@@ -5642,7 +5594,7 @@
       </c>
       <c r="I98" s="5" t="inlineStr">
         <is>
-          <t>rename = relabel only; merger = relabel + sum across ALL years; split and merge_split = flag only, never auto-apportion</t>
+          <t>rename = relabel only; merger = relabel and sum across ALL years; split and merge_split = flag only, never auto-apportion</t>
         </is>
       </c>
       <c r="J98" s="5" t="inlineStr">
@@ -5652,7 +5604,7 @@
       </c>
       <c r="K98" s="5" t="inlineStr">
         <is>
-          <t>The crosswalk relabels ALL years, not just post-change ones: sources are published under the geography current at PUBLICATION, so a year-conditional rule would orphan the absorbed county and undercount the survivor. This corrects the 8/31 scaffolding.</t>
+          <t>The crosswalk relabels all years, not just post-change ones: sources are published under the geography current at publication, so a year-conditional rule would orphan the absorbed county and undercount the survivor.</t>
         </is>
       </c>
     </row>
@@ -5665,7 +5617,7 @@
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>Change date, which reference confirms the row, and the verbatim Census wording</t>
+          <t>Change date, the reference that confirms the row, and the verbatim Census wording</t>
         </is>
       </c>
       <c r="D99" s="5" t="inlineStr">
@@ -5705,7 +5657,7 @@
       </c>
       <c r="K99" s="5" t="inlineStr">
         <is>
-          <t>Deliberately excluded: Alaska and the territories (CONUS + DC scope), CT's 2022 planning regions (not expressible as a rename/merger/split -- handled by 08a), and small boundary shifts where both geoids exist before and after. Only 51780 (1995) and 08014 (2001) land inside the good-collision-data window.</t>
+          <t>Excluded by scope: Alaska and the territories, CT's 2022 planning regions (not expressible as a rename/merger/split -- handled by 08a), and boundary shifts where both geoids exist before and after. Only 51780 (1995) and 08014 (2001) fall inside the collision window.</t>
         </is>
       </c>
     </row>
@@ -5723,7 +5675,7 @@
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>Number of months in this county-year whose PRISM day count did not match the calendar</t>
+          <t>Months in this county-year whose PRISM day count did not match the calendar</t>
         </is>
       </c>
       <c r="D100" s="5" t="inlineStr">
@@ -5753,7 +5705,7 @@
       </c>
       <c r="I100" s="5" t="inlineStr">
         <is>
-          <t>SECTION 1: gen byte temp = (is_incomplete == "True"); bysort geoid year: egen n_incomplete_months = total(temp); drop temp</t>
+          <t>SECTION 1: gen byte temp = (is_incomplete == "True"); bysort geoid year: egen n_incomplete_months = total(temp)</t>
         </is>
       </c>
       <c r="J100" s="5" t="inlineStr">
@@ -5781,47 +5733,42 @@
       </c>
       <c r="D101" s="5" t="inlineStr">
         <is>
-          <t>degrees C</t>
+          <t>numeric (double)</t>
         </is>
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t>numeric (double)</t>
+          <t>county-year</t>
         </is>
       </c>
       <c r="F101" s="5" t="inlineStr">
         <is>
-          <t>county-year</t>
+          <t>continuous, degrees C</t>
         </is>
       </c>
       <c r="G101" s="5" t="inlineStr">
         <is>
-          <t>continuous</t>
+          <t>mean_temp_c_m12/_m1/_m2</t>
         </is>
       </c>
       <c r="H101" s="5" t="inlineStr">
         <is>
-          <t>mean_temp_c_m12/_m1/_m2, from prism_derived_weather_vars.csv</t>
+          <t>1981-2025</t>
         </is>
       </c>
       <c r="I101" s="5" t="inlineStr">
         <is>
-          <t>1981-2025</t>
+          <t>SECTION 7: gen double mean_winter_temp = (L1.mean_temp_c_m12 + mean_temp_c_m1 + mean_temp_c_m2)/3, using the SECTION 6 xtset</t>
         </is>
       </c>
       <c r="J101" s="5" t="inlineStr">
         <is>
-          <t>SECTION 7: gen double mean_winter_temp = (L1.mean_temp_c_m12 + mean_temp_c_m1 + mean_temp_c_m2)/3, using the xtset declared in SECTION 6</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K101" s="5" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="L101" s="5" t="inlineStr">
-        <is>
-          <t>Built in the merge script, not in the estimation do-files, so every downstream script uses the identical construction. Its DJF window is NARROWER than the WSI's Dec 1 - Apr 30 window. Missing in the panel's first year (December of t-1 is out of sample). Recomputed independently by 09b rather than read back.</t>
+          <t>Built in the merge script, not the estimation do-files, so every downstream script uses the identical construction. Its DJF window is NARROWER than the WSI's Dec 1 - Apr 30. Missing in the panel's first year.</t>
         </is>
       </c>
     </row>
@@ -5839,47 +5786,42 @@
       </c>
       <c r="D102" s="5" t="inlineStr">
         <is>
-          <t>0/1 dummy</t>
+          <t>numeric (byte)</t>
         </is>
       </c>
       <c r="E102" s="5" t="inlineStr">
         <is>
-          <t>numeric (byte)</t>
+          <t>county-year</t>
         </is>
       </c>
       <c r="F102" s="5" t="inlineStr">
         <is>
-          <t>county-year</t>
+          <t>0/1; missing where mean_winter_temp is missing</t>
         </is>
       </c>
       <c r="G102" s="5" t="inlineStr">
         <is>
-          <t>0/1, missing where mean_winter_temp is missing</t>
+          <t>Derived from mean_winter_temp</t>
         </is>
       </c>
       <c r="H102" s="5" t="inlineStr">
         <is>
-          <t>Derived from mean_winter_temp</t>
+          <t>1981-2025</t>
         </is>
       </c>
       <c r="I102" s="5" t="inlineStr">
         <is>
-          <t>1981-2025</t>
+          <t>SECTION 7: bysort fips_num: egen the county's own mean and SD of mean_winter_temp over the full panel, then compare</t>
         </is>
       </c>
       <c r="J102" s="5" t="inlineStr">
         <is>
-          <t>SECTION 7: bysort fips_num: egen the county's own mean and SD of mean_winter_temp over the full panel, then compare</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K102" s="5" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="L102" s="5" t="inlineStr">
-        <is>
-          <t>'Local climatology' is each county's own 1981-2025 record (settled 9/5/26), so these are within-county anomalies, not cross-sectional. One-directional -- warm side only.</t>
+          <t>Within-county anomalies against each county's own 1981-2025 record, not cross-sectional. One-directional -- warm side only.</t>
         </is>
       </c>
     </row>
@@ -5922,7 +5864,7 @@
       </c>
       <c r="I103" s="5" t="inlineStr">
         <is>
-          <t>merge 1:1 geoid year, renamed rather than asserted/dropped -- a deliberate departure from the style guide's merge convention, settled 9/1/26. SECTION 8 exports diagnostics instead. The winter-severity merge is the exception: keep(master match), because an unmatched USING row would mean 06c and the weather spine disagree about the county-year universe.</t>
+          <t>merge 1:1 geoid year, renamed rather than asserted or dropped; SECTION 8 exports diagnostics instead. The winter-severity merge uses keep(master match), since an unmatched using row would mean 06c and the weather spine disagree about the county-year universe.</t>
         </is>
       </c>
       <c r="J103" s="5" t="inlineStr">
@@ -5939,7 +5881,7 @@
     <row r="105" ht="20" customHeight="1">
       <c r="A105" s="6" t="inlineStr">
         <is>
-          <t>OPEN QUESTIONS &amp; FLAGS -- WEATHER (codePYTHON 02a-06c)</t>
+          <t>KNOWN DATA ISSUES -- read before using these variables</t>
         </is>
       </c>
       <c r="B105" s="7" t="n"/>
@@ -5961,7 +5903,7 @@
       </c>
       <c r="B106" s="5" t="inlineStr">
         <is>
-          <t>PRISM daily-vs-composited discrepancy: compositing an ImageCollection with .sum()/.mean() and reducing once gives values ~1-2% off from reducing each day independently, even though both operations are linear. Root cause not diagnosed. Every script in the pipeline therefore reduces day-by-day and aggregates afterward -- keep it that way, and do not 'optimize' an extraction into a composite-then-reduce.</t>
+          <t>wsi_snow_days is near-degenerate across most of the eastern deer range. Kohn's 18in cutoff was calibrated on point station observations, while snow_depth here is an ERA5-Land grid-box average averaged again over a whole county. On the 1981 extract Wisconsin recorded 8 county-days &gt;=18in statewide and MN/IA/IL/PA none. winter_severity_index is therefore effectively wsi_cold_days over most of the study area; the 12in/8in variants exist so that can be shown rather than asserted.</t>
         </is>
       </c>
       <c r="C106" s="8" t="n"/>
@@ -5982,7 +5924,7 @@
       </c>
       <c r="B107" s="5" t="inlineStr">
         <is>
-          <t>TIGER/2018/Counties contains two separate features for 18 Wisconsin GEOIDs, so their daily rows are written twice, byte-for-byte identical. 05/06 drop byte-identical duplicates automatically and error if any non-key column disagrees. Harmless as observed, but it is a property of the source collection, not of our code.</t>
+          <t>geoid 25019 (Nantucket, MA) has no valid ERA5-Land land pixel inside the county polygon: 16,436 missing daily readings, mean_snow_depth missing, and every snow day-count 0 rather than missing. A Nantucket WSI of 0 is a data gap, not a mild winter.</t>
         </is>
       </c>
       <c r="C107" s="8" t="n"/>
@@ -6003,7 +5945,7 @@
       </c>
       <c r="B108" s="5" t="inlineStr">
         <is>
-          <t>wsi_snow_days is near-degenerate across most of the eastern deer range: Kohn's 18in cutoff was calibrated on point station observations, while snow_depth here is an ERA5-Land grid-box average averaged again over a whole county. On the 1981 extract Wisconsin recorded 8 county-days &gt;=18in statewide and MN/IA/IL/PA none. winter_severity_index is therefore effectively wsi_cold_days over most of the study area. The 12in/8in variants exist so this can be shown rather than asserted. Still open with the PI.</t>
+          <t>ERA5's tmin_c_mean/tmax_c_mean and the ERA5 derived-variable block duplicate PRISM's by design, and the base names collide. Rename before merging both into one panel.</t>
         </is>
       </c>
       <c r="C108" s="8" t="n"/>
@@ -6019,12 +5961,12 @@
     <row r="109" ht="42" customHeight="1">
       <c r="A109" s="4" t="inlineStr">
         <is>
-          <t>WEA-4</t>
+          <t>POP-1</t>
         </is>
       </c>
       <c r="B109" s="5" t="inlineStr">
         <is>
-          <t>06b_validate_ppt_total.py is NOT wired into _project_main.do and should not be until its failure mode changes: sys.exit(1) inside Stata's embedded interpreter raises SystemExit and halts the master script. Same applies to 07b. Also note that a bare 06b run checks PRISM only -- pass --dataset PRISM --dataset ERA5.</t>
+          <t>CT 2021-2025 has population totals but no age shares (40 county-years, age_flag set). Genuinely unavailable, not a build gap -- do not model them down.</t>
         </is>
       </c>
       <c r="C109" s="8" t="n"/>
@@ -6040,12 +5982,12 @@
     <row r="110" ht="42" customHeight="1">
       <c r="A110" s="4" t="inlineStr">
         <is>
-          <t>WEA-5</t>
+          <t>POP-2</t>
         </is>
       </c>
       <c r="B110" s="5" t="inlineStr">
         <is>
-          <t>The ground-truth case lists are hand-synced across 07e, 07f, 07g and 07h, and 07e's list has drifted from the others (different counties AND different years). Reconcile before trusting a cross-dataset PRISM-vs-ERA5-vs-station comparison.</t>
+          <t>Broomfield CO (08014) is missing before 2001 and its four parent counties carry a discontinuity flag at 2001. No apportionment was built: collisions for the area were filed under the parents too, so a back-apportioned denominator would produce a fake near-zero collision rate for two decades.</t>
         </is>
       </c>
       <c r="C110" s="8" t="n"/>
@@ -6061,12 +6003,12 @@
     <row r="111" ht="42" customHeight="1">
       <c r="A111" s="4" t="inlineStr">
         <is>
-          <t>WEA-6</t>
+          <t>POP-3</t>
         </is>
       </c>
       <c r="B111" s="5" t="inlineStr">
         <is>
-          <t>ERA5's tmin_c_mean/tmax_c_mean duplicate PRISM's tmin_mean/tmax_mean by design (ERA5 needs its own to serve as a robustness check). Confirm with the team that both are wanted downstream before anyone merges them into the same panel -- the base names collide.</t>
+          <t>2020-2025 is postcensal and provisional -- it will be revised once the 2030 census anchors it. 1981-2019 is intercensal and final. The 2020 row is the 4/1/2020 census count while every other year is a July 1 estimate (~0.2%).</t>
         </is>
       </c>
       <c r="C111" s="8" t="n"/>
@@ -6082,12 +6024,12 @@
     <row r="112" ht="42" customHeight="1">
       <c r="A112" s="4" t="inlineStr">
         <is>
-          <t>WEA-7</t>
+          <t>POP-4</t>
         </is>
       </c>
       <c r="B112" s="5" t="inlineStr">
         <is>
-          <t>geoid 25019 (Nantucket, MA) has no valid ERA5-Land land pixel inside the county polygon: 16,436 missing daily readings, mean_snow_depth missing, and every snow day-count 0 rather than missing. A Nantucket WSI of 0 is a data gap, not a mild winter.</t>
+          <t>The canonical panel is population_county_year_1981_2025.{csv,dta}, built on Kodama, and that is what SECTION 3 reads. Kodama also holds an older 1990-2025 pair; do not build against it.</t>
         </is>
       </c>
       <c r="C112" s="8" t="n"/>
@@ -6103,12 +6045,12 @@
     <row r="113" ht="42" customHeight="1">
       <c r="A113" s="4" t="inlineStr">
         <is>
-          <t>WEA-8</t>
+          <t>GEN-1</t>
         </is>
       </c>
       <c r="B113" s="5" t="inlineStr">
         <is>
-          <t>06c has not been run against the local dataCSV copy -- the Mac's prism_derived_weather_vars.csv is the 2020-2021 test slice and predates days_extremely_cold, and there is no local ERA5 derived file. It was verified on synthetic fixtures and against Kodama's panel.</t>
+          <t>Every monthly weather measure enters main_data_county_year.dta as 12 columns, &lt;var&gt;_m1 .. &lt;var&gt;_m12: 12 PRISM base variables = 144 columns, 5 ERA5 snow variables = 60 columns.</t>
         </is>
       </c>
       <c r="C113" s="8" t="n"/>
@@ -6121,32 +6063,36 @@
       <c r="J113" s="8" t="n"/>
       <c r="K113" s="8" t="n"/>
     </row>
-    <row r="114" ht="20" customHeight="1">
-      <c r="A114" s="6" t="inlineStr">
-        <is>
-          <t>OPEN QUESTIONS &amp; FLAGS -- POPULATION (codePYTHON 08a/08b)</t>
-        </is>
-      </c>
-      <c r="B114" s="7" t="n"/>
-      <c r="C114" s="7" t="n"/>
-      <c r="D114" s="7" t="n"/>
-      <c r="E114" s="7" t="n"/>
-      <c r="F114" s="7" t="n"/>
-      <c r="G114" s="7" t="n"/>
-      <c r="H114" s="7" t="n"/>
-      <c r="I114" s="7" t="n"/>
-      <c r="J114" s="7" t="n"/>
-      <c r="K114" s="7" t="n"/>
+    <row r="114" ht="42" customHeight="1">
+      <c r="A114" s="4" t="inlineStr">
+        <is>
+          <t>GEN-2</t>
+        </is>
+      </c>
+      <c r="B114" s="5" t="inlineStr">
+        <is>
+          <t>PRISM is the project's weather source for temperature and precipitation; ERA5-Land is a robustness check against it. ERA5 is merged into the main panel for its snow variables only.</t>
+        </is>
+      </c>
+      <c r="C114" s="8" t="n"/>
+      <c r="D114" s="8" t="n"/>
+      <c r="E114" s="8" t="n"/>
+      <c r="F114" s="8" t="n"/>
+      <c r="G114" s="8" t="n"/>
+      <c r="H114" s="8" t="n"/>
+      <c r="I114" s="8" t="n"/>
+      <c r="J114" s="8" t="n"/>
+      <c r="K114" s="8" t="n"/>
     </row>
     <row r="115" ht="42" customHeight="1">
       <c r="A115" s="4" t="inlineStr">
         <is>
-          <t>POP-1</t>
+          <t>GEN-3</t>
         </is>
       </c>
       <c r="B115" s="5" t="inlineStr">
         <is>
-          <t>08a's CT design is NOT ratified by the PI. The mechanism validates (169 towns -&gt; 8 counties, within 0.1% at 2015 and 2018), but the approach itself was never signed off. CT was raised on 9/1/26 and the answer that came back was about the Dorn PDF and the 1980s.</t>
+          <t>prism_county_month.csv and era5_county_month.csv (05) do not feed the merge -- they are the descriptive-exhibit panel. SECTION 1 reads prism_derived_weather_vars.csv (06), which recomputes monthly precipitation from the same dailies by a different route; 06b exists to catch the two drifting apart.</t>
         </is>
       </c>
       <c r="C115" s="8" t="n"/>
@@ -6159,276 +6105,18 @@
       <c r="J115" s="8" t="n"/>
       <c r="K115" s="8" t="n"/>
     </row>
-    <row r="116" ht="42" customHeight="1">
-      <c r="A116" s="4" t="inlineStr">
-        <is>
-          <t>POP-2</t>
-        </is>
-      </c>
-      <c r="B116" s="5" t="inlineStr">
-        <is>
-          <t>CT 2021-2025 has population totals but no age shares (40 county-years, age_flag set). Genuinely unavailable, not a build gap -- do not model them down.</t>
-        </is>
-      </c>
-      <c r="C116" s="8" t="n"/>
-      <c r="D116" s="8" t="n"/>
-      <c r="E116" s="8" t="n"/>
-      <c r="F116" s="8" t="n"/>
-      <c r="G116" s="8" t="n"/>
-      <c r="H116" s="8" t="n"/>
-      <c r="I116" s="8" t="n"/>
-      <c r="J116" s="8" t="n"/>
-      <c r="K116" s="8" t="n"/>
-    </row>
-    <row r="117" ht="42" customHeight="1">
-      <c r="A117" s="4" t="inlineStr">
-        <is>
-          <t>POP-3</t>
-        </is>
-      </c>
-      <c r="B117" s="5" t="inlineStr">
-        <is>
-          <t>Broomfield CO (08014) is left missing before 2001 and its four parent counties carry a discontinuity flag at 2001. No apportionment was built, deliberately: collisions for the area were filed under the parents too, so a back-apportioned denominator would produce a fake near-zero collision rate for two decades.</t>
-        </is>
-      </c>
-      <c r="C117" s="8" t="n"/>
-      <c r="D117" s="8" t="n"/>
-      <c r="E117" s="8" t="n"/>
-      <c r="F117" s="8" t="n"/>
-      <c r="G117" s="8" t="n"/>
-      <c r="H117" s="8" t="n"/>
-      <c r="I117" s="8" t="n"/>
-      <c r="J117" s="8" t="n"/>
-      <c r="K117" s="8" t="n"/>
-    </row>
-    <row r="118" ht="42" customHeight="1">
-      <c r="A118" s="4" t="inlineStr">
-        <is>
-          <t>POP-4</t>
-        </is>
-      </c>
-      <c r="B118" s="5" t="inlineStr">
-        <is>
-          <t>The 2020 row is the 4/1/2020 census count (from the 2010-2020 intercensal) while every other year is a July 1 estimate. ~0.2%, immaterial, but undocumented in the appendix and never put to the PI.</t>
-        </is>
-      </c>
-      <c r="C118" s="8" t="n"/>
-      <c r="D118" s="8" t="n"/>
-      <c r="E118" s="8" t="n"/>
-      <c r="F118" s="8" t="n"/>
-      <c r="G118" s="8" t="n"/>
-      <c r="H118" s="8" t="n"/>
-      <c r="I118" s="8" t="n"/>
-      <c r="J118" s="8" t="n"/>
-      <c r="K118" s="8" t="n"/>
-    </row>
-    <row r="119" ht="42" customHeight="1">
-      <c r="A119" s="4" t="inlineStr">
-        <is>
-          <t>POP-5</t>
-        </is>
-      </c>
-      <c r="B119" s="5" t="inlineStr">
-        <is>
-          <t>2020-2025 is POSTCENSAL and provisional -- it will be revised once the 2030 census anchors it. Everything 1981-2019 is intercensal and final.</t>
-        </is>
-      </c>
-      <c r="C119" s="8" t="n"/>
-      <c r="D119" s="8" t="n"/>
-      <c r="E119" s="8" t="n"/>
-      <c r="F119" s="8" t="n"/>
-      <c r="G119" s="8" t="n"/>
-      <c r="H119" s="8" t="n"/>
-      <c r="I119" s="8" t="n"/>
-      <c r="J119" s="8" t="n"/>
-      <c r="K119" s="8" t="n"/>
-    </row>
-    <row r="120" ht="42" customHeight="1">
-      <c r="A120" s="4" t="inlineStr">
-        <is>
-          <t>POP-6</t>
-        </is>
-      </c>
-      <c r="B120" s="5" t="inlineStr">
-        <is>
-          <t>The canonical panel is population_county_year_1981_2025.{csv,dta}, built on Kodama 9/9/26, and that is what SECTION 3 reads. The Mac's dataCSV/Population holds only the older 1990-2025 pair; Kodama holds both side by side. Do not build against the 1990-2025 file.</t>
-        </is>
-      </c>
-      <c r="C120" s="8" t="n"/>
-      <c r="D120" s="8" t="n"/>
-      <c r="E120" s="8" t="n"/>
-      <c r="F120" s="8" t="n"/>
-      <c r="G120" s="8" t="n"/>
-      <c r="H120" s="8" t="n"/>
-      <c r="I120" s="8" t="n"/>
-      <c r="J120" s="8" t="n"/>
-      <c r="K120" s="8" t="n"/>
-    </row>
-    <row r="121" ht="42" customHeight="1">
-      <c r="A121" s="4" t="inlineStr">
-        <is>
-          <t>POP-7</t>
-        </is>
-      </c>
-      <c r="B121" s="5" t="inlineStr">
-        <is>
-          <t>Run python3 codePYTHON/test_population_logic.py (66 offline checks, no network) before reviewing or extending 08a/08b.</t>
-        </is>
-      </c>
-      <c r="C121" s="8" t="n"/>
-      <c r="D121" s="8" t="n"/>
-      <c r="E121" s="8" t="n"/>
-      <c r="F121" s="8" t="n"/>
-      <c r="G121" s="8" t="n"/>
-      <c r="H121" s="8" t="n"/>
-      <c r="I121" s="8" t="n"/>
-      <c r="J121" s="8" t="n"/>
-      <c r="K121" s="8" t="n"/>
-    </row>
-    <row r="122" ht="20" customHeight="1">
-      <c r="A122" s="6" t="inlineStr">
-        <is>
-          <t>GENERAL</t>
-        </is>
-      </c>
-      <c r="B122" s="7" t="n"/>
-      <c r="C122" s="7" t="n"/>
-      <c r="D122" s="7" t="n"/>
-      <c r="E122" s="7" t="n"/>
-      <c r="F122" s="7" t="n"/>
-      <c r="G122" s="7" t="n"/>
-      <c r="H122" s="7" t="n"/>
-      <c r="I122" s="7" t="n"/>
-      <c r="J122" s="7" t="n"/>
-      <c r="K122" s="7" t="n"/>
-    </row>
-    <row r="123" ht="42" customHeight="1">
-      <c r="A123" s="4" t="inlineStr">
-        <is>
-          <t>GEN-1</t>
-        </is>
-      </c>
-      <c r="B123" s="5" t="inlineStr">
-        <is>
-          <t>Weather monthly measures enter main_data_county_year.dta as 12 columns each, &lt;var&gt;_m1 .. &lt;var&gt;_m12 (the _m suffix is a 9/5/26 call; Stata's own reshape produces a bare `mean_temp_c1`). 11 PRISM base variables plus ppt_total = 144 columns, 5 ERA5 snow variables = 60 columns.</t>
-        </is>
-      </c>
-      <c r="C123" s="8" t="n"/>
-      <c r="D123" s="8" t="n"/>
-      <c r="E123" s="8" t="n"/>
-      <c r="F123" s="8" t="n"/>
-      <c r="G123" s="8" t="n"/>
-      <c r="H123" s="8" t="n"/>
-      <c r="I123" s="8" t="n"/>
-      <c r="J123" s="8" t="n"/>
-      <c r="K123" s="8" t="n"/>
-    </row>
-    <row r="124" ht="42" customHeight="1">
-      <c r="A124" s="4" t="inlineStr">
-        <is>
-          <t>GEN-2</t>
-        </is>
-      </c>
-      <c r="B124" s="5" t="inlineStr">
-        <is>
-          <t>PRISM is the project's main weather dataset for temperature and precipitation; ERA5-Land is a robustness check against it, not a co-equal source. ERA5 is merged into the main panel for its snow variables only, which PRISM has no equivalent for.</t>
-        </is>
-      </c>
-      <c r="C124" s="8" t="n"/>
-      <c r="D124" s="8" t="n"/>
-      <c r="E124" s="8" t="n"/>
-      <c r="F124" s="8" t="n"/>
-      <c r="G124" s="8" t="n"/>
-      <c r="H124" s="8" t="n"/>
-      <c r="I124" s="8" t="n"/>
-      <c r="J124" s="8" t="n"/>
-      <c r="K124" s="8" t="n"/>
-    </row>
-    <row r="125" ht="42" customHeight="1">
-      <c r="A125" s="4" t="inlineStr">
-        <is>
-          <t>GEN-3</t>
-        </is>
-      </c>
-      <c r="B125" s="5" t="inlineStr">
-        <is>
-          <t>prism_county_month.csv / era5_county_month.csv (05) do NOT feed the merge -- they are the descriptive-exhibit panel (09a/09b). SECTION 1 reads prism_derived_weather_vars.csv (06). 06 computes monthly precipitation from the same dailies by a different route, and 06b exists to catch the two drifting apart.</t>
-        </is>
-      </c>
-      <c r="C125" s="8" t="n"/>
-      <c r="D125" s="8" t="n"/>
-      <c r="E125" s="8" t="n"/>
-      <c r="F125" s="8" t="n"/>
-      <c r="G125" s="8" t="n"/>
-      <c r="H125" s="8" t="n"/>
-      <c r="I125" s="8" t="n"/>
-      <c r="J125" s="8" t="n"/>
-      <c r="K125" s="8" t="n"/>
-    </row>
-    <row r="126" ht="42" customHeight="1">
-      <c r="A126" s="4" t="inlineStr">
-        <is>
-          <t>GEN-4</t>
-        </is>
-      </c>
-      <c r="B126" s="5" t="inlineStr">
-        <is>
-          <t>None of these scripts apply Stata variable labels at the CSV stage; labels are attached in build_main_data_county_year.do. Adding labels there that mirror the Description column here would let this dictionary be regenerated with `describe` instead of maintained by hand.</t>
-        </is>
-      </c>
-      <c r="C126" s="8" t="n"/>
-      <c r="D126" s="8" t="n"/>
-      <c r="E126" s="8" t="n"/>
-      <c r="F126" s="8" t="n"/>
-      <c r="G126" s="8" t="n"/>
-      <c r="H126" s="8" t="n"/>
-      <c r="I126" s="8" t="n"/>
-      <c r="J126" s="8" t="n"/>
-      <c r="K126" s="8" t="n"/>
-    </row>
-    <row r="127" ht="42" customHeight="1">
-      <c r="A127" s="4" t="inlineStr">
-        <is>
-          <t>GEN-5</t>
-        </is>
-      </c>
-      <c r="B127" s="5" t="inlineStr">
-        <is>
-          <t>Seven of the codePYTHON scripts are what _project_main.do actually runs: 05, 06, 06c, 08a, 08b, 09a, 09b. Everything else is a test, a spot-check or a one-off, run by hand.</t>
-        </is>
-      </c>
-      <c r="C127" s="8" t="n"/>
-      <c r="D127" s="8" t="n"/>
-      <c r="E127" s="8" t="n"/>
-      <c r="F127" s="8" t="n"/>
-      <c r="G127" s="8" t="n"/>
-      <c r="H127" s="8" t="n"/>
-      <c r="I127" s="8" t="n"/>
-      <c r="J127" s="8" t="n"/>
-      <c r="K127" s="8" t="n"/>
-    </row>
   </sheetData>
-  <mergeCells count="21">
+  <mergeCells count="11">
+    <mergeCell ref="B114:K114"/>
     <mergeCell ref="B108:K108"/>
-    <mergeCell ref="B118:K118"/>
-    <mergeCell ref="B127:K127"/>
-    <mergeCell ref="B124:K124"/>
+    <mergeCell ref="B107:K107"/>
     <mergeCell ref="B110:K110"/>
-    <mergeCell ref="B123:K123"/>
-    <mergeCell ref="B126:K126"/>
+    <mergeCell ref="B115:K115"/>
+    <mergeCell ref="A2:K2"/>
     <mergeCell ref="B106:K106"/>
     <mergeCell ref="B113:K113"/>
     <mergeCell ref="B109:K109"/>
-    <mergeCell ref="B125:K125"/>
-    <mergeCell ref="B121:K121"/>
-    <mergeCell ref="B115:K115"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="B117:K117"/>
     <mergeCell ref="B111:K111"/>
-    <mergeCell ref="B120:K120"/>
-    <mergeCell ref="B107:K107"/>
-    <mergeCell ref="B119:K119"/>
-    <mergeCell ref="B116:K116"/>
     <mergeCell ref="B112:K112"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>